<commit_message>
Add gitignore and RP2350A, RP2350B, RP2354A, and RP2354B components
</commit_message>
<xml_diff>
--- a/Moonlight_Library.xlsx
+++ b/Moonlight_Library.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Altium\Libraries\Moonlight_Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mani\Documents\Projects\altium\libraries\Moonlight_Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5189623B-7403-45C7-A1C7-3B1446389525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602AE9D9-9C10-4EAD-8B08-B00CD7404CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="905" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16305" yWindow="6900" windowWidth="16410" windowHeight="14145" tabRatio="905" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capacitors Polar" sheetId="3" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5766" uniqueCount="1336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5814" uniqueCount="1346">
   <si>
     <t>Symbol Ref</t>
   </si>
@@ -4058,6 +4058,36 @@
   </si>
   <si>
     <t>X5R, 6.3V</t>
+  </si>
+  <si>
+    <t>RP235xB</t>
+  </si>
+  <si>
+    <t>RP2350A</t>
+  </si>
+  <si>
+    <t>RP2354A</t>
+  </si>
+  <si>
+    <t>RP2350B</t>
+  </si>
+  <si>
+    <t>RP2354B</t>
+  </si>
+  <si>
+    <t>Dual Core 150 MHz ARM-M33 Microcontroller</t>
+  </si>
+  <si>
+    <t>Dual Core 150 MHz ARM-M33 Microcontroller with 2 MB Flash</t>
+  </si>
+  <si>
+    <t>QFN-60 (7x7)</t>
+  </si>
+  <si>
+    <t>QFN-80 (10x10)</t>
+  </si>
+  <si>
+    <t>RP235xA</t>
   </si>
 </sst>
 </file>
@@ -20097,7 +20127,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B93A8C-0336-4B42-880D-67109C66C120}">
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" style="6" bestFit="1" customWidth="1"/>
@@ -20210,28 +20240,25 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>569</v>
-      </c>
-      <c r="B3" t="s">
-        <v>570</v>
+        <v>1345</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>1345</v>
       </c>
       <c r="C3" t="s">
-        <v>570</v>
-      </c>
-      <c r="D3" t="s">
-        <v>569</v>
+        <v>1343</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>1345</v>
       </c>
       <c r="E3" t="s">
-        <v>568</v>
-      </c>
-      <c r="F3" t="s">
-        <v>572</v>
+        <v>13</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>1337</v>
       </c>
       <c r="G3" t="s">
-        <v>568</v>
-      </c>
-      <c r="H3" t="s">
-        <v>572</v>
+        <v>48</v>
       </c>
       <c r="I3" t="s">
         <v>7</v>
@@ -20240,39 +20267,36 @@
         <v>16</v>
       </c>
       <c r="M3" t="s">
-        <v>571</v>
+        <v>1341</v>
       </c>
       <c r="O3" t="s">
         <v>520</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="6" t="s">
         <v>896</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="B4" t="s">
-        <v>576</v>
+        <v>1345</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>1345</v>
       </c>
       <c r="C4" t="s">
-        <v>576</v>
-      </c>
-      <c r="D4" t="s">
-        <v>573</v>
+        <v>1343</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>1345</v>
       </c>
       <c r="E4" t="s">
-        <v>575</v>
-      </c>
-      <c r="F4" t="s">
-        <v>573</v>
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>1338</v>
       </c>
       <c r="G4" t="s">
         <v>48</v>
-      </c>
-      <c r="H4" t="s">
-        <v>577</v>
       </c>
       <c r="I4" t="s">
         <v>7</v>
@@ -20281,39 +20305,36 @@
         <v>16</v>
       </c>
       <c r="M4" t="s">
-        <v>578</v>
+        <v>1342</v>
       </c>
       <c r="O4" t="s">
         <v>520</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="6" t="s">
         <v>896</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>574</v>
+        <v>1336</v>
       </c>
       <c r="B5" t="s">
-        <v>574</v>
+        <v>1336</v>
       </c>
       <c r="C5" t="s">
-        <v>580</v>
+        <v>1344</v>
       </c>
       <c r="D5" t="s">
-        <v>574</v>
+        <v>1336</v>
       </c>
       <c r="E5" t="s">
-        <v>575</v>
+        <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>574</v>
+        <v>1339</v>
       </c>
       <c r="G5" t="s">
         <v>48</v>
-      </c>
-      <c r="H5" t="s">
-        <v>579</v>
       </c>
       <c r="I5" t="s">
         <v>7</v>
@@ -20322,33 +20343,33 @@
         <v>16</v>
       </c>
       <c r="M5" t="s">
-        <v>581</v>
+        <v>1341</v>
       </c>
       <c r="O5" t="s">
         <v>520</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="6" t="s">
         <v>896</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>1006</v>
+        <v>1336</v>
       </c>
       <c r="B6" t="s">
-        <v>584</v>
+        <v>1336</v>
       </c>
       <c r="C6" t="s">
-        <v>584</v>
+        <v>1344</v>
       </c>
       <c r="D6" t="s">
-        <v>1006</v>
+        <v>1336</v>
       </c>
       <c r="E6" t="s">
-        <v>751</v>
+        <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>1006</v>
+        <v>1340</v>
       </c>
       <c r="G6" t="s">
         <v>48</v>
@@ -20360,39 +20381,39 @@
         <v>16</v>
       </c>
       <c r="M6" t="s">
-        <v>1007</v>
+        <v>1342</v>
       </c>
       <c r="O6" t="s">
         <v>520</v>
       </c>
-      <c r="P6" t="s">
-        <v>895</v>
+      <c r="P6" s="6" t="s">
+        <v>896</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>1015</v>
+        <v>569</v>
       </c>
       <c r="B7" t="s">
-        <v>1015</v>
+        <v>570</v>
       </c>
       <c r="C7" t="s">
-        <v>1018</v>
+        <v>570</v>
       </c>
       <c r="D7" t="s">
-        <v>1015</v>
+        <v>569</v>
       </c>
       <c r="E7" t="s">
-        <v>585</v>
+        <v>568</v>
       </c>
       <c r="F7" t="s">
-        <v>1015</v>
+        <v>572</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>568</v>
       </c>
       <c r="H7" t="s">
-        <v>1016</v>
+        <v>572</v>
       </c>
       <c r="I7" t="s">
         <v>7</v>
@@ -20401,39 +20422,39 @@
         <v>16</v>
       </c>
       <c r="M7" t="s">
-        <v>1017</v>
+        <v>571</v>
       </c>
       <c r="O7" t="s">
-        <v>583</v>
+        <v>520</v>
       </c>
       <c r="P7" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="B8" t="s">
-        <v>602</v>
+        <v>576</v>
       </c>
       <c r="C8" t="s">
-        <v>603</v>
+        <v>576</v>
       </c>
       <c r="D8" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="E8" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
       <c r="F8" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="G8" t="s">
         <v>48</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>587</v>
+      <c r="H8" t="s">
+        <v>577</v>
       </c>
       <c r="I8" t="s">
         <v>7</v>
@@ -20442,39 +20463,39 @@
         <v>16</v>
       </c>
       <c r="M8" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="O8" t="s">
-        <v>583</v>
+        <v>520</v>
       </c>
       <c r="P8" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>514</v>
+        <v>574</v>
       </c>
       <c r="B9" t="s">
-        <v>514</v>
+        <v>574</v>
       </c>
       <c r="C9" t="s">
-        <v>539</v>
+        <v>580</v>
       </c>
       <c r="D9" t="s">
-        <v>514</v>
+        <v>574</v>
       </c>
       <c r="E9" t="s">
-        <v>524</v>
+        <v>575</v>
       </c>
       <c r="F9" t="s">
-        <v>514</v>
+        <v>574</v>
       </c>
       <c r="G9" t="s">
         <v>48</v>
       </c>
       <c r="H9" t="s">
-        <v>530</v>
+        <v>579</v>
       </c>
       <c r="I9" t="s">
         <v>7</v>
@@ -20483,39 +20504,36 @@
         <v>16</v>
       </c>
       <c r="M9" t="s">
-        <v>554</v>
+        <v>581</v>
       </c>
       <c r="O9" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="P9" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>515</v>
+        <v>1006</v>
       </c>
       <c r="B10" t="s">
-        <v>549</v>
+        <v>584</v>
       </c>
       <c r="C10" t="s">
-        <v>531</v>
+        <v>584</v>
       </c>
       <c r="D10" t="s">
-        <v>515</v>
+        <v>1006</v>
       </c>
       <c r="E10" t="s">
-        <v>524</v>
+        <v>751</v>
       </c>
       <c r="F10" t="s">
-        <v>515</v>
+        <v>1006</v>
       </c>
       <c r="G10" t="s">
         <v>48</v>
-      </c>
-      <c r="H10" t="s">
-        <v>533</v>
       </c>
       <c r="I10" t="s">
         <v>7</v>
@@ -20524,42 +20542,39 @@
         <v>16</v>
       </c>
       <c r="M10" t="s">
-        <v>553</v>
-      </c>
-      <c r="N10" t="s">
-        <v>414</v>
+        <v>1007</v>
       </c>
       <c r="O10" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="P10" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>547</v>
+        <v>1015</v>
       </c>
       <c r="B11" t="s">
-        <v>549</v>
+        <v>1015</v>
       </c>
       <c r="C11" t="s">
-        <v>531</v>
+        <v>1018</v>
       </c>
       <c r="D11" t="s">
-        <v>547</v>
+        <v>1015</v>
       </c>
       <c r="E11" t="s">
-        <v>524</v>
+        <v>585</v>
       </c>
       <c r="F11" t="s">
-        <v>547</v>
+        <v>1015</v>
       </c>
       <c r="G11" t="s">
         <v>48</v>
       </c>
       <c r="H11" t="s">
-        <v>550</v>
+        <v>1016</v>
       </c>
       <c r="I11" t="s">
         <v>7</v>
@@ -20568,39 +20583,39 @@
         <v>16</v>
       </c>
       <c r="M11" t="s">
-        <v>553</v>
+        <v>1017</v>
       </c>
       <c r="O11" t="s">
-        <v>521</v>
+        <v>583</v>
       </c>
       <c r="P11" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>548</v>
+        <v>582</v>
       </c>
       <c r="B12" t="s">
-        <v>548</v>
+        <v>602</v>
       </c>
       <c r="C12" t="s">
-        <v>555</v>
+        <v>603</v>
       </c>
       <c r="D12" t="s">
-        <v>548</v>
+        <v>582</v>
       </c>
       <c r="E12" t="s">
-        <v>524</v>
+        <v>585</v>
       </c>
       <c r="F12" t="s">
-        <v>548</v>
+        <v>582</v>
       </c>
       <c r="G12" t="s">
         <v>48</v>
       </c>
-      <c r="H12" t="s">
-        <v>551</v>
+      <c r="H12" s="4" t="s">
+        <v>587</v>
       </c>
       <c r="I12" t="s">
         <v>7</v>
@@ -20609,10 +20624,10 @@
         <v>16</v>
       </c>
       <c r="M12" t="s">
-        <v>552</v>
+        <v>586</v>
       </c>
       <c r="O12" t="s">
-        <v>521</v>
+        <v>583</v>
       </c>
       <c r="P12" t="s">
         <v>895</v>
@@ -20620,28 +20635,28 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B13" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C13" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="D13" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="E13" t="s">
         <v>524</v>
       </c>
       <c r="F13" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="G13" t="s">
         <v>48</v>
       </c>
       <c r="H13" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="I13" t="s">
         <v>7</v>
@@ -20650,39 +20665,39 @@
         <v>16</v>
       </c>
       <c r="M13" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="O13" t="s">
         <v>521</v>
       </c>
       <c r="P13" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B14" t="s">
-        <v>517</v>
+        <v>549</v>
       </c>
       <c r="C14" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="D14" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="E14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F14" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="G14" t="s">
         <v>48</v>
       </c>
       <c r="H14" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="I14" t="s">
         <v>7</v>
@@ -20691,7 +20706,10 @@
         <v>16</v>
       </c>
       <c r="M14" t="s">
-        <v>544</v>
+        <v>553</v>
+      </c>
+      <c r="N14" t="s">
+        <v>414</v>
       </c>
       <c r="O14" t="s">
         <v>521</v>
@@ -20702,28 +20720,28 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
       <c r="B15" t="s">
-        <v>518</v>
+        <v>549</v>
       </c>
       <c r="C15" t="s">
-        <v>540</v>
+        <v>531</v>
       </c>
       <c r="D15" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
       <c r="E15" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="F15" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
       <c r="G15" t="s">
         <v>48</v>
       </c>
       <c r="H15" t="s">
-        <v>538</v>
+        <v>550</v>
       </c>
       <c r="I15" t="s">
         <v>7</v>
@@ -20732,7 +20750,7 @@
         <v>16</v>
       </c>
       <c r="M15" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="O15" t="s">
         <v>521</v>
@@ -20743,28 +20761,28 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>523</v>
+        <v>548</v>
       </c>
       <c r="B16" t="s">
-        <v>523</v>
+        <v>548</v>
       </c>
       <c r="C16" t="s">
-        <v>532</v>
+        <v>555</v>
       </c>
       <c r="D16" t="s">
-        <v>523</v>
+        <v>548</v>
       </c>
       <c r="E16" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="F16" t="s">
-        <v>523</v>
+        <v>548</v>
       </c>
       <c r="G16" t="s">
         <v>48</v>
       </c>
       <c r="H16" t="s">
-        <v>529</v>
+        <v>551</v>
       </c>
       <c r="I16" t="s">
         <v>7</v>
@@ -20773,39 +20791,39 @@
         <v>16</v>
       </c>
       <c r="M16" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="O16" t="s">
         <v>521</v>
       </c>
       <c r="P16" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="B17" t="s">
-        <v>542</v>
+        <v>516</v>
       </c>
       <c r="C17" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="D17" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="E17" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="F17" t="s">
-        <v>522</v>
+        <v>516</v>
       </c>
       <c r="G17" t="s">
         <v>48</v>
       </c>
       <c r="H17" t="s">
-        <v>541</v>
+        <v>535</v>
       </c>
       <c r="I17" t="s">
         <v>7</v>
@@ -20814,7 +20832,7 @@
         <v>16</v>
       </c>
       <c r="M17" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="O17" t="s">
         <v>521</v>
@@ -20825,28 +20843,28 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>854</v>
+        <v>517</v>
       </c>
       <c r="B18" t="s">
-        <v>855</v>
+        <v>517</v>
       </c>
       <c r="C18" t="s">
-        <v>855</v>
+        <v>536</v>
       </c>
       <c r="D18" t="s">
-        <v>856</v>
+        <v>517</v>
       </c>
       <c r="E18" t="s">
-        <v>857</v>
+        <v>525</v>
       </c>
       <c r="F18" t="s">
-        <v>856</v>
+        <v>517</v>
       </c>
       <c r="G18" t="s">
-        <v>858</v>
+        <v>48</v>
       </c>
       <c r="H18" t="s">
-        <v>859</v>
+        <v>537</v>
       </c>
       <c r="I18" t="s">
         <v>7</v>
@@ -20855,39 +20873,39 @@
         <v>16</v>
       </c>
       <c r="M18" t="s">
-        <v>860</v>
+        <v>544</v>
       </c>
       <c r="O18" t="s">
         <v>521</v>
       </c>
       <c r="P18" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>1034</v>
+        <v>518</v>
       </c>
       <c r="B19" t="s">
-        <v>1034</v>
+        <v>518</v>
       </c>
       <c r="C19" t="s">
-        <v>1034</v>
+        <v>540</v>
       </c>
       <c r="D19" t="s">
-        <v>1034</v>
+        <v>518</v>
       </c>
       <c r="E19" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F19" t="s">
-        <v>1034</v>
+        <v>518</v>
       </c>
       <c r="G19" t="s">
         <v>48</v>
       </c>
       <c r="H19" t="s">
-        <v>1035</v>
+        <v>538</v>
       </c>
       <c r="I19" t="s">
         <v>7</v>
@@ -20896,42 +20914,39 @@
         <v>16</v>
       </c>
       <c r="M19" t="s">
-        <v>1036</v>
-      </c>
-      <c r="N19" t="s">
-        <v>414</v>
+        <v>544</v>
       </c>
       <c r="O19" t="s">
         <v>521</v>
       </c>
       <c r="P19" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>588</v>
+        <v>523</v>
       </c>
       <c r="B20" t="s">
-        <v>584</v>
+        <v>523</v>
       </c>
       <c r="C20" t="s">
-        <v>584</v>
+        <v>532</v>
       </c>
       <c r="D20" t="s">
-        <v>589</v>
+        <v>523</v>
       </c>
       <c r="E20" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F20" t="s">
-        <v>589</v>
+        <v>523</v>
       </c>
       <c r="G20" t="s">
         <v>48</v>
       </c>
       <c r="H20" t="s">
-        <v>590</v>
+        <v>529</v>
       </c>
       <c r="I20" t="s">
         <v>7</v>
@@ -20940,10 +20955,10 @@
         <v>16</v>
       </c>
       <c r="M20" t="s">
-        <v>599</v>
+        <v>546</v>
       </c>
       <c r="O20" t="s">
-        <v>597</v>
+        <v>521</v>
       </c>
       <c r="P20" t="s">
         <v>896</v>
@@ -20951,28 +20966,28 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>591</v>
+        <v>522</v>
       </c>
       <c r="B21" t="s">
-        <v>602</v>
+        <v>542</v>
       </c>
       <c r="C21" t="s">
-        <v>603</v>
+        <v>542</v>
       </c>
       <c r="D21" t="s">
-        <v>592</v>
+        <v>522</v>
       </c>
       <c r="E21" t="s">
-        <v>594</v>
+        <v>527</v>
       </c>
       <c r="F21" t="s">
-        <v>592</v>
+        <v>522</v>
       </c>
       <c r="G21" t="s">
         <v>48</v>
       </c>
       <c r="H21" t="s">
-        <v>593</v>
+        <v>541</v>
       </c>
       <c r="I21" t="s">
         <v>7</v>
@@ -20981,10 +20996,10 @@
         <v>16</v>
       </c>
       <c r="M21" t="s">
-        <v>598</v>
+        <v>545</v>
       </c>
       <c r="O21" t="s">
-        <v>597</v>
+        <v>521</v>
       </c>
       <c r="P21" t="s">
         <v>896</v>
@@ -20992,28 +21007,28 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>601</v>
+        <v>854</v>
       </c>
       <c r="B22" t="s">
-        <v>584</v>
+        <v>855</v>
       </c>
       <c r="C22" t="s">
-        <v>584</v>
+        <v>855</v>
       </c>
       <c r="D22" t="s">
-        <v>595</v>
+        <v>856</v>
       </c>
       <c r="E22" t="s">
-        <v>527</v>
+        <v>857</v>
       </c>
       <c r="F22" t="s">
-        <v>595</v>
+        <v>856</v>
       </c>
       <c r="G22" t="s">
-        <v>48</v>
+        <v>858</v>
       </c>
       <c r="H22" t="s">
-        <v>596</v>
+        <v>859</v>
       </c>
       <c r="I22" t="s">
         <v>7</v>
@@ -21022,10 +21037,10 @@
         <v>16</v>
       </c>
       <c r="M22" t="s">
-        <v>600</v>
+        <v>860</v>
       </c>
       <c r="O22" t="s">
-        <v>597</v>
+        <v>521</v>
       </c>
       <c r="P22" t="s">
         <v>895</v>
@@ -21033,28 +21048,28 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>1253</v>
+        <v>1034</v>
       </c>
       <c r="B23" t="s">
-        <v>1255</v>
+        <v>1034</v>
       </c>
       <c r="C23" t="s">
-        <v>1254</v>
+        <v>1034</v>
       </c>
       <c r="D23" t="s">
-        <v>1255</v>
+        <v>1034</v>
       </c>
       <c r="E23" t="s">
-        <v>1207</v>
+        <v>527</v>
       </c>
       <c r="F23" t="s">
-        <v>1255</v>
+        <v>1034</v>
       </c>
       <c r="G23" t="s">
         <v>48</v>
       </c>
       <c r="H23" t="s">
-        <v>1256</v>
+        <v>1035</v>
       </c>
       <c r="I23" t="s">
         <v>7</v>
@@ -21063,10 +21078,13 @@
         <v>16</v>
       </c>
       <c r="M23" t="s">
-        <v>1257</v>
+        <v>1036</v>
+      </c>
+      <c r="N23" t="s">
+        <v>414</v>
       </c>
       <c r="O23" t="s">
-        <v>597</v>
+        <v>521</v>
       </c>
       <c r="P23" t="s">
         <v>895</v>
@@ -21074,28 +21092,28 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>1275</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>1275</v>
+        <v>588</v>
+      </c>
+      <c r="B24" t="s">
+        <v>584</v>
       </c>
       <c r="C24" t="s">
-        <v>1276</v>
+        <v>584</v>
       </c>
       <c r="D24" t="s">
-        <v>1277</v>
+        <v>589</v>
       </c>
       <c r="E24" t="s">
-        <v>1207</v>
+        <v>527</v>
       </c>
       <c r="F24" t="s">
-        <v>1277</v>
+        <v>589</v>
       </c>
       <c r="G24" t="s">
         <v>48</v>
       </c>
       <c r="H24" t="s">
-        <v>1278</v>
+        <v>590</v>
       </c>
       <c r="I24" t="s">
         <v>7</v>
@@ -21104,39 +21122,39 @@
         <v>16</v>
       </c>
       <c r="M24" t="s">
-        <v>1279</v>
+        <v>599</v>
       </c>
       <c r="O24" t="s">
-        <v>1274</v>
+        <v>597</v>
       </c>
       <c r="P24" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>868</v>
+        <v>591</v>
       </c>
       <c r="B25" t="s">
-        <v>869</v>
+        <v>602</v>
       </c>
       <c r="C25" t="s">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="D25" t="s">
-        <v>870</v>
+        <v>592</v>
       </c>
       <c r="E25" t="s">
-        <v>751</v>
+        <v>594</v>
       </c>
       <c r="F25" t="s">
-        <v>870</v>
+        <v>592</v>
       </c>
       <c r="G25" t="s">
         <v>48</v>
       </c>
       <c r="H25" t="s">
-        <v>871</v>
+        <v>593</v>
       </c>
       <c r="I25" t="s">
         <v>7</v>
@@ -21145,39 +21163,39 @@
         <v>16</v>
       </c>
       <c r="M25" t="s">
-        <v>873</v>
+        <v>598</v>
       </c>
       <c r="O25" t="s">
-        <v>872</v>
+        <v>597</v>
       </c>
       <c r="P25" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="B26" t="s">
-        <v>609</v>
+        <v>584</v>
       </c>
       <c r="C26" t="s">
-        <v>609</v>
+        <v>584</v>
       </c>
       <c r="D26" t="s">
-        <v>606</v>
+        <v>595</v>
       </c>
       <c r="E26" t="s">
-        <v>608</v>
+        <v>527</v>
       </c>
       <c r="F26" t="s">
-        <v>606</v>
+        <v>595</v>
       </c>
       <c r="G26" t="s">
         <v>48</v>
       </c>
       <c r="H26" t="s">
-        <v>607</v>
+        <v>596</v>
       </c>
       <c r="I26" t="s">
         <v>7</v>
@@ -21186,39 +21204,39 @@
         <v>16</v>
       </c>
       <c r="M26" t="s">
-        <v>1217</v>
+        <v>600</v>
       </c>
       <c r="O26" t="s">
-        <v>610</v>
+        <v>597</v>
       </c>
       <c r="P26" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>613</v>
+        <v>1253</v>
       </c>
       <c r="B27" t="s">
-        <v>615</v>
+        <v>1255</v>
       </c>
       <c r="C27" t="s">
-        <v>615</v>
+        <v>1254</v>
       </c>
       <c r="D27" t="s">
-        <v>613</v>
+        <v>1255</v>
       </c>
       <c r="E27" t="s">
-        <v>614</v>
+        <v>1207</v>
       </c>
       <c r="F27" t="s">
-        <v>613</v>
+        <v>1255</v>
       </c>
       <c r="G27" t="s">
         <v>48</v>
       </c>
       <c r="H27" t="s">
-        <v>612</v>
+        <v>1256</v>
       </c>
       <c r="I27" t="s">
         <v>7</v>
@@ -21227,10 +21245,10 @@
         <v>16</v>
       </c>
       <c r="M27" t="s">
-        <v>1022</v>
+        <v>1257</v>
       </c>
       <c r="O27" t="s">
-        <v>610</v>
+        <v>597</v>
       </c>
       <c r="P27" t="s">
         <v>895</v>
@@ -21238,28 +21256,28 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>1019</v>
-      </c>
-      <c r="B28" t="s">
-        <v>718</v>
+        <v>1275</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>1275</v>
       </c>
       <c r="C28" t="s">
-        <v>718</v>
+        <v>1276</v>
       </c>
       <c r="D28" t="s">
-        <v>1019</v>
+        <v>1277</v>
       </c>
       <c r="E28" t="s">
-        <v>719</v>
+        <v>1207</v>
       </c>
       <c r="F28" t="s">
-        <v>1019</v>
+        <v>1277</v>
       </c>
       <c r="G28" t="s">
         <v>48</v>
       </c>
       <c r="H28" t="s">
-        <v>1020</v>
+        <v>1278</v>
       </c>
       <c r="I28" t="s">
         <v>7</v>
@@ -21268,51 +21286,51 @@
         <v>16</v>
       </c>
       <c r="M28" t="s">
-        <v>1021</v>
+        <v>1279</v>
       </c>
       <c r="O28" t="s">
-        <v>610</v>
+        <v>1274</v>
       </c>
       <c r="P28" t="s">
         <v>895</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
-        <v>7805</v>
+      <c r="A29" s="6" t="s">
+        <v>868</v>
       </c>
       <c r="B29" t="s">
-        <v>1079</v>
+        <v>869</v>
       </c>
       <c r="C29" t="s">
-        <v>1079</v>
+        <v>869</v>
       </c>
       <c r="D29" t="s">
-        <v>1080</v>
+        <v>870</v>
       </c>
       <c r="E29" t="s">
-        <v>703</v>
+        <v>751</v>
       </c>
       <c r="F29" t="s">
-        <v>1080</v>
+        <v>870</v>
       </c>
       <c r="G29" t="s">
         <v>48</v>
       </c>
       <c r="H29" t="s">
-        <v>1081</v>
+        <v>871</v>
       </c>
       <c r="I29" t="s">
         <v>7</v>
       </c>
       <c r="J29" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M29" t="s">
-        <v>1082</v>
+        <v>873</v>
       </c>
       <c r="O29" t="s">
-        <v>610</v>
+        <v>872</v>
       </c>
       <c r="P29" t="s">
         <v>895</v>
@@ -21320,78 +21338,78 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>1097</v>
+        <v>606</v>
       </c>
       <c r="B30" t="s">
-        <v>1098</v>
+        <v>609</v>
       </c>
       <c r="C30" t="s">
-        <v>1098</v>
+        <v>609</v>
       </c>
       <c r="D30" t="s">
-        <v>1099</v>
+        <v>606</v>
       </c>
       <c r="E30" t="s">
-        <v>525</v>
+        <v>608</v>
       </c>
       <c r="F30" t="s">
-        <v>1099</v>
+        <v>606</v>
       </c>
       <c r="G30" t="s">
         <v>48</v>
       </c>
       <c r="H30" t="s">
-        <v>1100</v>
+        <v>607</v>
       </c>
       <c r="I30" t="s">
         <v>7</v>
       </c>
       <c r="J30" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M30" t="s">
-        <v>1101</v>
+        <v>1217</v>
       </c>
       <c r="O30" t="s">
         <v>610</v>
       </c>
       <c r="P30" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>1208</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="G31" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="B31" t="s">
+        <v>615</v>
+      </c>
+      <c r="C31" t="s">
+        <v>615</v>
+      </c>
+      <c r="D31" t="s">
+        <v>613</v>
+      </c>
+      <c r="E31" t="s">
+        <v>614</v>
+      </c>
+      <c r="F31" t="s">
+        <v>613</v>
+      </c>
+      <c r="G31" t="s">
         <v>48</v>
       </c>
       <c r="H31" t="s">
-        <v>1203</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J31" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="I31" t="s">
+        <v>7</v>
+      </c>
+      <c r="J31" t="s">
         <v>16</v>
       </c>
       <c r="M31" t="s">
-        <v>1218</v>
+        <v>1022</v>
       </c>
       <c r="O31" t="s">
         <v>610</v>
@@ -21402,37 +21420,37 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1219</v>
+        <v>1019</v>
       </c>
       <c r="B32" t="s">
-        <v>1219</v>
+        <v>718</v>
       </c>
       <c r="C32" t="s">
-        <v>1039</v>
+        <v>718</v>
       </c>
       <c r="D32" t="s">
-        <v>1214</v>
+        <v>1019</v>
       </c>
       <c r="E32" t="s">
-        <v>527</v>
+        <v>719</v>
       </c>
       <c r="F32" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G32" s="6" t="s">
+        <v>1019</v>
+      </c>
+      <c r="G32" t="s">
         <v>48</v>
       </c>
       <c r="H32" t="s">
-        <v>1215</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J32" s="6" t="s">
+        <v>1020</v>
+      </c>
+      <c r="I32" t="s">
+        <v>7</v>
+      </c>
+      <c r="J32" t="s">
         <v>16</v>
       </c>
       <c r="M32" t="s">
-        <v>1216</v>
+        <v>1021</v>
       </c>
       <c r="O32" t="s">
         <v>610</v>
@@ -21442,38 +21460,38 @@
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>1213</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>1213</v>
+      <c r="A33" s="6">
+        <v>7805</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1079</v>
       </c>
       <c r="C33" t="s">
-        <v>1204</v>
+        <v>1079</v>
       </c>
       <c r="D33" t="s">
-        <v>1205</v>
+        <v>1080</v>
       </c>
       <c r="E33" t="s">
-        <v>1207</v>
+        <v>703</v>
       </c>
       <c r="F33" t="s">
-        <v>1205</v>
-      </c>
-      <c r="G33" s="6" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G33" t="s">
         <v>48</v>
       </c>
       <c r="H33" t="s">
-        <v>1209</v>
-      </c>
-      <c r="I33" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J33" s="6" t="s">
-        <v>16</v>
+        <v>1081</v>
+      </c>
+      <c r="I33" t="s">
+        <v>7</v>
+      </c>
+      <c r="J33" t="s">
+        <v>8</v>
       </c>
       <c r="M33" t="s">
-        <v>1211</v>
+        <v>1082</v>
       </c>
       <c r="O33" t="s">
         <v>610</v>
@@ -21484,37 +21502,37 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>1213</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>1213</v>
+        <v>1097</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1098</v>
       </c>
       <c r="C34" t="s">
-        <v>1204</v>
+        <v>1098</v>
       </c>
       <c r="D34" t="s">
-        <v>1206</v>
+        <v>1099</v>
       </c>
       <c r="E34" t="s">
-        <v>1207</v>
+        <v>525</v>
       </c>
       <c r="F34" t="s">
-        <v>1206</v>
-      </c>
-      <c r="G34" s="6" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G34" t="s">
         <v>48</v>
       </c>
       <c r="H34" t="s">
-        <v>1210</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>16</v>
+        <v>1100</v>
+      </c>
+      <c r="I34" t="s">
+        <v>7</v>
+      </c>
+      <c r="J34" t="s">
+        <v>8</v>
       </c>
       <c r="M34" t="s">
-        <v>1212</v>
+        <v>1101</v>
       </c>
       <c r="O34" t="s">
         <v>610</v>
@@ -21525,40 +21543,40 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B35" t="s">
-        <v>1038</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1039</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1040</v>
-      </c>
-      <c r="E35" t="s">
-        <v>751</v>
-      </c>
-      <c r="F35" t="s">
-        <v>1040</v>
-      </c>
-      <c r="G35" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>1208</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="G35" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H35" t="s">
-        <v>1041</v>
-      </c>
-      <c r="I35" t="s">
-        <v>7</v>
-      </c>
-      <c r="J35" t="s">
+        <v>1203</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J35" s="6" t="s">
         <v>16</v>
       </c>
       <c r="M35" t="s">
-        <v>1042</v>
+        <v>1218</v>
       </c>
       <c r="O35" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P35" t="s">
         <v>895</v>
@@ -21566,40 +21584,40 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1037</v>
+        <v>1219</v>
       </c>
       <c r="B36" t="s">
-        <v>1038</v>
+        <v>1219</v>
       </c>
       <c r="C36" t="s">
         <v>1039</v>
       </c>
       <c r="D36" t="s">
-        <v>1044</v>
+        <v>1214</v>
       </c>
       <c r="E36" t="s">
-        <v>751</v>
+        <v>527</v>
       </c>
       <c r="F36" t="s">
-        <v>1044</v>
-      </c>
-      <c r="G36" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G36" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H36" t="s">
-        <v>1045</v>
-      </c>
-      <c r="I36" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36" t="s">
+        <v>1215</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J36" s="6" t="s">
         <v>16</v>
       </c>
       <c r="M36" t="s">
-        <v>1046</v>
+        <v>1216</v>
       </c>
       <c r="O36" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P36" t="s">
         <v>895</v>
@@ -21607,40 +21625,40 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1038</v>
+        <v>1213</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>1213</v>
       </c>
       <c r="C37" t="s">
-        <v>1039</v>
+        <v>1204</v>
       </c>
       <c r="D37" t="s">
-        <v>1047</v>
+        <v>1205</v>
       </c>
       <c r="E37" t="s">
-        <v>751</v>
+        <v>1207</v>
       </c>
       <c r="F37" t="s">
-        <v>1047</v>
-      </c>
-      <c r="G37" t="s">
+        <v>1205</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H37" t="s">
-        <v>1048</v>
-      </c>
-      <c r="I37" t="s">
-        <v>7</v>
-      </c>
-      <c r="J37" t="s">
+        <v>1209</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J37" s="6" t="s">
         <v>16</v>
       </c>
       <c r="M37" t="s">
-        <v>1049</v>
+        <v>1211</v>
       </c>
       <c r="O37" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P37" t="s">
         <v>895</v>
@@ -21648,40 +21666,40 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B38" t="s">
-        <v>1038</v>
+        <v>1213</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>1213</v>
       </c>
       <c r="C38" t="s">
-        <v>1039</v>
+        <v>1204</v>
       </c>
       <c r="D38" t="s">
-        <v>1050</v>
+        <v>1206</v>
       </c>
       <c r="E38" t="s">
-        <v>751</v>
+        <v>1207</v>
       </c>
       <c r="F38" t="s">
-        <v>1050</v>
-      </c>
-      <c r="G38" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G38" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H38" t="s">
-        <v>1051</v>
-      </c>
-      <c r="I38" t="s">
-        <v>7</v>
-      </c>
-      <c r="J38" t="s">
+        <v>1210</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J38" s="6" t="s">
         <v>16</v>
       </c>
       <c r="M38" t="s">
-        <v>1052</v>
+        <v>1212</v>
       </c>
       <c r="O38" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P38" t="s">
         <v>895</v>
@@ -21698,19 +21716,19 @@
         <v>1039</v>
       </c>
       <c r="D39" t="s">
-        <v>1053</v>
+        <v>1040</v>
       </c>
       <c r="E39" t="s">
         <v>751</v>
       </c>
       <c r="F39" t="s">
-        <v>1053</v>
+        <v>1040</v>
       </c>
       <c r="G39" t="s">
         <v>48</v>
       </c>
       <c r="H39" t="s">
-        <v>1054</v>
+        <v>1041</v>
       </c>
       <c r="I39" t="s">
         <v>7</v>
@@ -21719,7 +21737,7 @@
         <v>16</v>
       </c>
       <c r="M39" t="s">
-        <v>1055</v>
+        <v>1042</v>
       </c>
       <c r="O39" t="s">
         <v>1043</v>
@@ -21739,19 +21757,19 @@
         <v>1039</v>
       </c>
       <c r="D40" t="s">
-        <v>1056</v>
+        <v>1044</v>
       </c>
       <c r="E40" t="s">
         <v>751</v>
       </c>
       <c r="F40" t="s">
-        <v>1056</v>
+        <v>1044</v>
       </c>
       <c r="G40" t="s">
         <v>48</v>
       </c>
       <c r="H40" t="s">
-        <v>1057</v>
+        <v>1045</v>
       </c>
       <c r="I40" t="s">
         <v>7</v>
@@ -21760,7 +21778,7 @@
         <v>16</v>
       </c>
       <c r="M40" t="s">
-        <v>1058</v>
+        <v>1046</v>
       </c>
       <c r="O40" t="s">
         <v>1043</v>
@@ -21780,19 +21798,19 @@
         <v>1039</v>
       </c>
       <c r="D41" t="s">
-        <v>1059</v>
+        <v>1047</v>
       </c>
       <c r="E41" t="s">
         <v>751</v>
       </c>
       <c r="F41" t="s">
-        <v>1059</v>
+        <v>1047</v>
       </c>
       <c r="G41" t="s">
         <v>48</v>
       </c>
       <c r="H41" t="s">
-        <v>1060</v>
+        <v>1048</v>
       </c>
       <c r="I41" t="s">
         <v>7</v>
@@ -21801,7 +21819,7 @@
         <v>16</v>
       </c>
       <c r="M41" t="s">
-        <v>1061</v>
+        <v>1049</v>
       </c>
       <c r="O41" t="s">
         <v>1043</v>
@@ -21821,19 +21839,19 @@
         <v>1039</v>
       </c>
       <c r="D42" t="s">
-        <v>1062</v>
+        <v>1050</v>
       </c>
       <c r="E42" t="s">
         <v>751</v>
       </c>
       <c r="F42" t="s">
-        <v>1062</v>
+        <v>1050</v>
       </c>
       <c r="G42" t="s">
         <v>48</v>
       </c>
       <c r="H42" t="s">
-        <v>1063</v>
+        <v>1051</v>
       </c>
       <c r="I42" t="s">
         <v>7</v>
@@ -21842,7 +21860,7 @@
         <v>16</v>
       </c>
       <c r="M42" t="s">
-        <v>1064</v>
+        <v>1052</v>
       </c>
       <c r="O42" t="s">
         <v>1043</v>
@@ -21862,19 +21880,19 @@
         <v>1039</v>
       </c>
       <c r="D43" t="s">
-        <v>1065</v>
+        <v>1053</v>
       </c>
       <c r="E43" t="s">
         <v>751</v>
       </c>
       <c r="F43" t="s">
-        <v>1065</v>
+        <v>1053</v>
       </c>
       <c r="G43" t="s">
         <v>48</v>
       </c>
       <c r="H43" t="s">
-        <v>1066</v>
+        <v>1054</v>
       </c>
       <c r="I43" t="s">
         <v>7</v>
@@ -21883,7 +21901,7 @@
         <v>16</v>
       </c>
       <c r="M43" t="s">
-        <v>1067</v>
+        <v>1055</v>
       </c>
       <c r="O43" t="s">
         <v>1043</v>
@@ -21903,19 +21921,19 @@
         <v>1039</v>
       </c>
       <c r="D44" t="s">
-        <v>1068</v>
+        <v>1056</v>
       </c>
       <c r="E44" t="s">
         <v>751</v>
       </c>
       <c r="F44" t="s">
-        <v>1068</v>
+        <v>1056</v>
       </c>
       <c r="G44" t="s">
         <v>48</v>
       </c>
       <c r="H44" t="s">
-        <v>1069</v>
+        <v>1057</v>
       </c>
       <c r="I44" t="s">
         <v>7</v>
@@ -21924,7 +21942,7 @@
         <v>16</v>
       </c>
       <c r="M44" t="s">
-        <v>1070</v>
+        <v>1058</v>
       </c>
       <c r="O44" t="s">
         <v>1043</v>
@@ -21935,28 +21953,28 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>611</v>
+        <v>1037</v>
       </c>
       <c r="B45" t="s">
-        <v>611</v>
+        <v>1038</v>
       </c>
       <c r="C45" t="s">
-        <v>617</v>
+        <v>1039</v>
       </c>
       <c r="D45" t="s">
-        <v>611</v>
+        <v>1059</v>
       </c>
       <c r="E45" t="s">
-        <v>525</v>
+        <v>751</v>
       </c>
       <c r="F45" t="s">
-        <v>611</v>
+        <v>1059</v>
       </c>
       <c r="G45" t="s">
         <v>48</v>
       </c>
       <c r="H45" t="s">
-        <v>616</v>
+        <v>1060</v>
       </c>
       <c r="I45" t="s">
         <v>7</v>
@@ -21965,39 +21983,39 @@
         <v>16</v>
       </c>
       <c r="M45" t="s">
-        <v>878</v>
+        <v>1061</v>
       </c>
       <c r="O45" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P45" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>875</v>
+        <v>1037</v>
       </c>
       <c r="B46" t="s">
-        <v>875</v>
+        <v>1038</v>
       </c>
       <c r="C46" t="s">
-        <v>877</v>
+        <v>1039</v>
       </c>
       <c r="D46" t="s">
-        <v>874</v>
+        <v>1062</v>
       </c>
       <c r="E46" t="s">
-        <v>527</v>
+        <v>751</v>
       </c>
       <c r="F46" t="s">
-        <v>874</v>
+        <v>1062</v>
       </c>
       <c r="G46" t="s">
         <v>48</v>
       </c>
       <c r="H46" t="s">
-        <v>876</v>
+        <v>1063</v>
       </c>
       <c r="I46" t="s">
         <v>7</v>
@@ -22006,10 +22024,10 @@
         <v>16</v>
       </c>
       <c r="M46" t="s">
-        <v>879</v>
+        <v>1064</v>
       </c>
       <c r="O46" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P46" t="s">
         <v>895</v>
@@ -22017,28 +22035,28 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>887</v>
+        <v>1037</v>
       </c>
       <c r="B47" t="s">
-        <v>886</v>
+        <v>1038</v>
       </c>
       <c r="C47" t="s">
-        <v>886</v>
+        <v>1039</v>
       </c>
       <c r="D47" t="s">
-        <v>880</v>
+        <v>1065</v>
       </c>
       <c r="E47" t="s">
-        <v>527</v>
+        <v>751</v>
       </c>
       <c r="F47" t="s">
-        <v>880</v>
+        <v>1065</v>
       </c>
       <c r="G47" t="s">
         <v>48</v>
       </c>
       <c r="H47" t="s">
-        <v>881</v>
+        <v>1066</v>
       </c>
       <c r="I47" t="s">
         <v>7</v>
@@ -22047,10 +22065,10 @@
         <v>16</v>
       </c>
       <c r="M47" t="s">
-        <v>882</v>
+        <v>1067</v>
       </c>
       <c r="O47" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P47" t="s">
         <v>895</v>
@@ -22058,28 +22076,28 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>888</v>
+        <v>1037</v>
       </c>
       <c r="B48" t="s">
-        <v>886</v>
+        <v>1038</v>
       </c>
       <c r="C48" t="s">
-        <v>886</v>
+        <v>1039</v>
       </c>
       <c r="D48" t="s">
-        <v>883</v>
+        <v>1068</v>
       </c>
       <c r="E48" t="s">
-        <v>527</v>
+        <v>751</v>
       </c>
       <c r="F48" t="s">
-        <v>883</v>
+        <v>1068</v>
       </c>
       <c r="G48" t="s">
         <v>48</v>
       </c>
       <c r="H48" t="s">
-        <v>884</v>
+        <v>1069</v>
       </c>
       <c r="I48" t="s">
         <v>7</v>
@@ -22088,10 +22106,10 @@
         <v>16</v>
       </c>
       <c r="M48" t="s">
-        <v>885</v>
+        <v>1070</v>
       </c>
       <c r="O48" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P48" t="s">
         <v>895</v>
@@ -22099,28 +22117,28 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>861</v>
+        <v>611</v>
       </c>
       <c r="B49" t="s">
-        <v>861</v>
+        <v>611</v>
       </c>
       <c r="C49" t="s">
-        <v>862</v>
+        <v>617</v>
       </c>
       <c r="D49" t="s">
-        <v>863</v>
+        <v>611</v>
       </c>
       <c r="E49" t="s">
-        <v>864</v>
+        <v>525</v>
       </c>
       <c r="F49" t="s">
-        <v>863</v>
+        <v>611</v>
       </c>
       <c r="G49" t="s">
         <v>48</v>
       </c>
       <c r="H49" t="s">
-        <v>865</v>
+        <v>616</v>
       </c>
       <c r="I49" t="s">
         <v>7</v>
@@ -22129,51 +22147,51 @@
         <v>16</v>
       </c>
       <c r="M49" t="s">
-        <v>866</v>
+        <v>878</v>
       </c>
       <c r="O49" t="s">
-        <v>867</v>
+        <v>618</v>
       </c>
       <c r="P49" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>930</v>
+        <v>875</v>
       </c>
       <c r="B50" t="s">
-        <v>615</v>
+        <v>875</v>
       </c>
       <c r="C50" t="s">
-        <v>615</v>
+        <v>877</v>
       </c>
       <c r="D50" t="s">
-        <v>931</v>
+        <v>874</v>
       </c>
       <c r="E50" t="s">
         <v>527</v>
       </c>
       <c r="F50" t="s">
-        <v>931</v>
+        <v>874</v>
       </c>
       <c r="G50" t="s">
         <v>48</v>
       </c>
       <c r="H50" t="s">
-        <v>932</v>
+        <v>876</v>
       </c>
       <c r="I50" t="s">
         <v>7</v>
       </c>
       <c r="J50" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M50" t="s">
-        <v>934</v>
+        <v>879</v>
       </c>
       <c r="O50" t="s">
-        <v>933</v>
+        <v>618</v>
       </c>
       <c r="P50" t="s">
         <v>895</v>
@@ -22181,28 +22199,28 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>1111</v>
+        <v>887</v>
       </c>
       <c r="B51" t="s">
-        <v>1111</v>
+        <v>886</v>
       </c>
       <c r="C51" t="s">
-        <v>1110</v>
+        <v>886</v>
       </c>
       <c r="D51" t="s">
-        <v>1112</v>
+        <v>880</v>
       </c>
       <c r="E51" t="s">
-        <v>1106</v>
+        <v>527</v>
       </c>
       <c r="F51" t="s">
-        <v>1116</v>
+        <v>880</v>
       </c>
       <c r="G51" t="s">
         <v>48</v>
       </c>
       <c r="H51" t="s">
-        <v>1120</v>
+        <v>881</v>
       </c>
       <c r="I51" t="s">
         <v>7</v>
@@ -22211,10 +22229,10 @@
         <v>16</v>
       </c>
       <c r="M51" t="s">
-        <v>1109</v>
+        <v>882</v>
       </c>
       <c r="O51" t="s">
-        <v>565</v>
+        <v>618</v>
       </c>
       <c r="P51" t="s">
         <v>895</v>
@@ -22222,28 +22240,28 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>1111</v>
+        <v>888</v>
       </c>
       <c r="B52" t="s">
-        <v>1111</v>
+        <v>886</v>
       </c>
       <c r="C52" t="s">
-        <v>1110</v>
+        <v>886</v>
       </c>
       <c r="D52" t="s">
-        <v>1113</v>
+        <v>883</v>
       </c>
       <c r="E52" t="s">
-        <v>1106</v>
+        <v>527</v>
       </c>
       <c r="F52" t="s">
-        <v>1117</v>
+        <v>883</v>
       </c>
       <c r="G52" t="s">
         <v>48</v>
       </c>
       <c r="H52" t="s">
-        <v>1121</v>
+        <v>884</v>
       </c>
       <c r="I52" t="s">
         <v>7</v>
@@ -22252,10 +22270,10 @@
         <v>16</v>
       </c>
       <c r="M52" t="s">
-        <v>1109</v>
+        <v>885</v>
       </c>
       <c r="O52" t="s">
-        <v>565</v>
+        <v>618</v>
       </c>
       <c r="P52" t="s">
         <v>895</v>
@@ -22263,28 +22281,28 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>1111</v>
+        <v>861</v>
       </c>
       <c r="B53" t="s">
-        <v>1111</v>
+        <v>861</v>
       </c>
       <c r="C53" t="s">
-        <v>1110</v>
+        <v>862</v>
       </c>
       <c r="D53" t="s">
-        <v>1114</v>
+        <v>863</v>
       </c>
       <c r="E53" t="s">
-        <v>1106</v>
+        <v>864</v>
       </c>
       <c r="F53" t="s">
-        <v>1118</v>
+        <v>863</v>
       </c>
       <c r="G53" t="s">
         <v>48</v>
       </c>
       <c r="H53" t="s">
-        <v>1122</v>
+        <v>865</v>
       </c>
       <c r="I53" t="s">
         <v>7</v>
@@ -22293,10 +22311,10 @@
         <v>16</v>
       </c>
       <c r="M53" t="s">
-        <v>1109</v>
+        <v>866</v>
       </c>
       <c r="O53" t="s">
-        <v>565</v>
+        <v>867</v>
       </c>
       <c r="P53" t="s">
         <v>895</v>
@@ -22304,40 +22322,40 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>1111</v>
+        <v>930</v>
       </c>
       <c r="B54" t="s">
-        <v>1111</v>
+        <v>615</v>
       </c>
       <c r="C54" t="s">
-        <v>1110</v>
+        <v>615</v>
       </c>
       <c r="D54" t="s">
-        <v>1115</v>
+        <v>931</v>
       </c>
       <c r="E54" t="s">
-        <v>1106</v>
+        <v>527</v>
       </c>
       <c r="F54" t="s">
-        <v>1119</v>
+        <v>931</v>
       </c>
       <c r="G54" t="s">
         <v>48</v>
       </c>
       <c r="H54" t="s">
-        <v>1123</v>
+        <v>932</v>
       </c>
       <c r="I54" t="s">
         <v>7</v>
       </c>
       <c r="J54" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M54" t="s">
-        <v>1109</v>
+        <v>934</v>
       </c>
       <c r="O54" t="s">
-        <v>565</v>
+        <v>933</v>
       </c>
       <c r="P54" t="s">
         <v>895</v>
@@ -22354,19 +22372,19 @@
         <v>1110</v>
       </c>
       <c r="D55" t="s">
-        <v>1105</v>
+        <v>1112</v>
       </c>
       <c r="E55" t="s">
         <v>1106</v>
       </c>
       <c r="F55" t="s">
-        <v>1107</v>
+        <v>1116</v>
       </c>
       <c r="G55" t="s">
         <v>48</v>
       </c>
       <c r="H55" t="s">
-        <v>1108</v>
+        <v>1120</v>
       </c>
       <c r="I55" t="s">
         <v>7</v>
@@ -22386,28 +22404,28 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>556</v>
+        <v>1111</v>
       </c>
       <c r="B56" t="s">
-        <v>562</v>
+        <v>1111</v>
       </c>
       <c r="C56" t="s">
-        <v>562</v>
+        <v>1110</v>
       </c>
       <c r="D56" t="s">
-        <v>556</v>
+        <v>1113</v>
       </c>
       <c r="E56" t="s">
-        <v>557</v>
+        <v>1106</v>
       </c>
       <c r="F56" t="s">
-        <v>556</v>
+        <v>1117</v>
       </c>
       <c r="G56" t="s">
-        <v>558</v>
+        <v>48</v>
       </c>
       <c r="H56" t="s">
-        <v>561</v>
+        <v>1121</v>
       </c>
       <c r="I56" t="s">
         <v>7</v>
@@ -22416,39 +22434,39 @@
         <v>16</v>
       </c>
       <c r="M56" t="s">
-        <v>566</v>
+        <v>1109</v>
       </c>
       <c r="O56" t="s">
         <v>565</v>
       </c>
       <c r="P56" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>559</v>
+        <v>1111</v>
       </c>
       <c r="B57" t="s">
-        <v>564</v>
+        <v>1111</v>
       </c>
       <c r="C57" t="s">
-        <v>564</v>
+        <v>1110</v>
       </c>
       <c r="D57" t="s">
-        <v>559</v>
+        <v>1114</v>
       </c>
       <c r="E57" t="s">
-        <v>557</v>
+        <v>1106</v>
       </c>
       <c r="F57" t="s">
-        <v>559</v>
+        <v>1118</v>
       </c>
       <c r="G57" t="s">
         <v>48</v>
       </c>
       <c r="H57" t="s">
-        <v>560</v>
+        <v>1122</v>
       </c>
       <c r="I57" t="s">
         <v>7</v>
@@ -22457,39 +22475,39 @@
         <v>16</v>
       </c>
       <c r="M57" t="s">
-        <v>567</v>
+        <v>1109</v>
       </c>
       <c r="O57" t="s">
         <v>565</v>
       </c>
       <c r="P57" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>1246</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>1246</v>
+        <v>1111</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1111</v>
       </c>
       <c r="C58" t="s">
-        <v>1248</v>
+        <v>1110</v>
       </c>
       <c r="D58" t="s">
-        <v>1244</v>
+        <v>1115</v>
       </c>
       <c r="E58" t="s">
-        <v>527</v>
+        <v>1106</v>
       </c>
       <c r="F58" t="s">
-        <v>1244</v>
+        <v>1119</v>
       </c>
       <c r="G58" t="s">
         <v>48</v>
       </c>
       <c r="H58" t="s">
-        <v>1245</v>
+        <v>1123</v>
       </c>
       <c r="I58" t="s">
         <v>7</v>
@@ -22498,12 +22516,176 @@
         <v>16</v>
       </c>
       <c r="M58" t="s">
+        <v>1109</v>
+      </c>
+      <c r="O58" t="s">
+        <v>565</v>
+      </c>
+      <c r="P58" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E59" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F59" t="s">
+        <v>1107</v>
+      </c>
+      <c r="G59" t="s">
+        <v>48</v>
+      </c>
+      <c r="H59" t="s">
+        <v>1108</v>
+      </c>
+      <c r="I59" t="s">
+        <v>7</v>
+      </c>
+      <c r="J59" t="s">
+        <v>16</v>
+      </c>
+      <c r="M59" t="s">
+        <v>1109</v>
+      </c>
+      <c r="O59" t="s">
+        <v>565</v>
+      </c>
+      <c r="P59" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="B60" t="s">
+        <v>562</v>
+      </c>
+      <c r="C60" t="s">
+        <v>562</v>
+      </c>
+      <c r="D60" t="s">
+        <v>556</v>
+      </c>
+      <c r="E60" t="s">
+        <v>557</v>
+      </c>
+      <c r="F60" t="s">
+        <v>556</v>
+      </c>
+      <c r="G60" t="s">
+        <v>558</v>
+      </c>
+      <c r="H60" t="s">
+        <v>561</v>
+      </c>
+      <c r="I60" t="s">
+        <v>7</v>
+      </c>
+      <c r="J60" t="s">
+        <v>16</v>
+      </c>
+      <c r="M60" t="s">
+        <v>566</v>
+      </c>
+      <c r="O60" t="s">
+        <v>565</v>
+      </c>
+      <c r="P60" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="B61" t="s">
+        <v>564</v>
+      </c>
+      <c r="C61" t="s">
+        <v>564</v>
+      </c>
+      <c r="D61" t="s">
+        <v>559</v>
+      </c>
+      <c r="E61" t="s">
+        <v>557</v>
+      </c>
+      <c r="F61" t="s">
+        <v>559</v>
+      </c>
+      <c r="G61" t="s">
+        <v>48</v>
+      </c>
+      <c r="H61" t="s">
+        <v>560</v>
+      </c>
+      <c r="I61" t="s">
+        <v>7</v>
+      </c>
+      <c r="J61" t="s">
+        <v>16</v>
+      </c>
+      <c r="M61" t="s">
+        <v>567</v>
+      </c>
+      <c r="O61" t="s">
+        <v>565</v>
+      </c>
+      <c r="P61" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1244</v>
+      </c>
+      <c r="E62" t="s">
+        <v>527</v>
+      </c>
+      <c r="F62" t="s">
+        <v>1244</v>
+      </c>
+      <c r="G62" t="s">
+        <v>48</v>
+      </c>
+      <c r="H62" t="s">
+        <v>1245</v>
+      </c>
+      <c r="I62" t="s">
+        <v>7</v>
+      </c>
+      <c r="J62" t="s">
+        <v>16</v>
+      </c>
+      <c r="M62" t="s">
         <v>1247</v>
       </c>
-      <c r="O58" t="s">
+      <c r="O62" t="s">
         <v>1243</v>
       </c>
-      <c r="P58" t="s">
+      <c r="P62" t="s">
         <v>895</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix RP235xx status and add 1.1V LDO
</commit_message>
<xml_diff>
--- a/Moonlight_Library.xlsx
+++ b/Moonlight_Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mani\Documents\Projects\altium\libraries\Moonlight_Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602AE9D9-9C10-4EAD-8B08-B00CD7404CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6551DF-3A19-4A3F-8774-F2A28783B9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16305" yWindow="6900" windowWidth="16410" windowHeight="14145" tabRatio="905" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="905" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capacitors Polar" sheetId="3" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5814" uniqueCount="1346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5847" uniqueCount="1366">
   <si>
     <t>Symbol Ref</t>
   </si>
@@ -4088,6 +4088,66 @@
   </si>
   <si>
     <t>RP235xA</t>
+  </si>
+  <si>
+    <t>1.1V 700mA LDO linear regulator, 1.9-6V input</t>
+  </si>
+  <si>
+    <t>893-XC6222B111MR-GCT-ND</t>
+  </si>
+  <si>
+    <t>XC6222B111MR-G</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>12V</t>
+  </si>
+  <si>
+    <t>1V</t>
+  </si>
+  <si>
+    <t>3.3V</t>
+  </si>
+  <si>
+    <t>1.1V</t>
+  </si>
+  <si>
+    <t>1.8V</t>
+  </si>
+  <si>
+    <t>1.024V</t>
+  </si>
+  <si>
+    <t>1.250V</t>
+  </si>
+  <si>
+    <t>1.800V</t>
+  </si>
+  <si>
+    <t>2.048V</t>
+  </si>
+  <si>
+    <t>2.500V</t>
+  </si>
+  <si>
+    <t>3.000V</t>
+  </si>
+  <si>
+    <t>3.300V</t>
+  </si>
+  <si>
+    <t>4.096V</t>
+  </si>
+  <si>
+    <t>4.500V</t>
+  </si>
+  <si>
+    <t>5.000V</t>
+  </si>
+  <si>
+    <t>0.6-34.2V</t>
   </si>
 </sst>
 </file>
@@ -20127,7 +20187,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B93A8C-0336-4B42-880D-67109C66C120}">
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" style="6" bestFit="1" customWidth="1"/>
@@ -20140,7 +20200,7 @@
     <col min="9" max="9" width="6.5703125" customWidth="1"/>
     <col min="10" max="10" width="12.140625" customWidth="1"/>
     <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" customWidth="1"/>
     <col min="13" max="13" width="71.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="34.5703125" customWidth="1"/>
     <col min="15" max="15" width="16.5703125" customWidth="1"/>
@@ -20273,7 +20333,7 @@
         <v>520</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -20311,7 +20371,7 @@
         <v>520</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -20349,7 +20409,7 @@
         <v>520</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -20387,7 +20447,7 @@
         <v>520</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -21367,6 +21427,9 @@
       <c r="J30" t="s">
         <v>16</v>
       </c>
+      <c r="L30" t="s">
+        <v>1349</v>
+      </c>
       <c r="M30" t="s">
         <v>1217</v>
       </c>
@@ -21408,6 +21471,9 @@
       <c r="J31" t="s">
         <v>16</v>
       </c>
+      <c r="L31" t="s">
+        <v>1352</v>
+      </c>
       <c r="M31" t="s">
         <v>1022</v>
       </c>
@@ -21420,28 +21486,28 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1019</v>
+        <v>1348</v>
       </c>
       <c r="B32" t="s">
-        <v>718</v>
+        <v>615</v>
       </c>
       <c r="C32" t="s">
-        <v>718</v>
+        <v>615</v>
       </c>
       <c r="D32" t="s">
-        <v>1019</v>
+        <v>1348</v>
       </c>
       <c r="E32" t="s">
-        <v>719</v>
+        <v>614</v>
       </c>
       <c r="F32" t="s">
-        <v>1019</v>
+        <v>1348</v>
       </c>
       <c r="G32" t="s">
         <v>48</v>
       </c>
       <c r="H32" t="s">
-        <v>1020</v>
+        <v>1347</v>
       </c>
       <c r="I32" t="s">
         <v>7</v>
@@ -21449,49 +21515,55 @@
       <c r="J32" t="s">
         <v>16</v>
       </c>
+      <c r="L32" t="s">
+        <v>1353</v>
+      </c>
       <c r="M32" t="s">
-        <v>1021</v>
+        <v>1346</v>
       </c>
       <c r="O32" t="s">
         <v>610</v>
       </c>
       <c r="P32" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
-        <v>7805</v>
+      <c r="A33" s="6" t="s">
+        <v>1019</v>
       </c>
       <c r="B33" t="s">
-        <v>1079</v>
+        <v>718</v>
       </c>
       <c r="C33" t="s">
-        <v>1079</v>
+        <v>718</v>
       </c>
       <c r="D33" t="s">
-        <v>1080</v>
+        <v>1019</v>
       </c>
       <c r="E33" t="s">
-        <v>703</v>
+        <v>719</v>
       </c>
       <c r="F33" t="s">
-        <v>1080</v>
+        <v>1019</v>
       </c>
       <c r="G33" t="s">
         <v>48</v>
       </c>
       <c r="H33" t="s">
-        <v>1081</v>
+        <v>1020</v>
       </c>
       <c r="I33" t="s">
         <v>7</v>
       </c>
       <c r="J33" t="s">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="L33" t="s">
+        <v>1352</v>
       </c>
       <c r="M33" t="s">
-        <v>1082</v>
+        <v>1021</v>
       </c>
       <c r="O33" t="s">
         <v>610</v>
@@ -21501,29 +21573,29 @@
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>1097</v>
+      <c r="A34" s="6">
+        <v>7805</v>
       </c>
       <c r="B34" t="s">
-        <v>1098</v>
+        <v>1079</v>
       </c>
       <c r="C34" t="s">
-        <v>1098</v>
+        <v>1079</v>
       </c>
       <c r="D34" t="s">
-        <v>1099</v>
+        <v>1080</v>
       </c>
       <c r="E34" t="s">
-        <v>525</v>
+        <v>703</v>
       </c>
       <c r="F34" t="s">
-        <v>1099</v>
+        <v>1080</v>
       </c>
       <c r="G34" t="s">
         <v>48</v>
       </c>
       <c r="H34" t="s">
-        <v>1100</v>
+        <v>1081</v>
       </c>
       <c r="I34" t="s">
         <v>7</v>
@@ -21531,8 +21603,11 @@
       <c r="J34" t="s">
         <v>8</v>
       </c>
+      <c r="L34" t="s">
+        <v>1349</v>
+      </c>
       <c r="M34" t="s">
-        <v>1101</v>
+        <v>1082</v>
       </c>
       <c r="O34" t="s">
         <v>610</v>
@@ -21543,37 +21618,40 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>1208</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="G35" s="6" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E35" t="s">
+        <v>525</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G35" t="s">
         <v>48</v>
       </c>
       <c r="H35" t="s">
-        <v>1203</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>16</v>
+        <v>1100</v>
+      </c>
+      <c r="I35" t="s">
+        <v>7</v>
+      </c>
+      <c r="J35" t="s">
+        <v>8</v>
+      </c>
+      <c r="L35" t="s">
+        <v>1350</v>
       </c>
       <c r="M35" t="s">
-        <v>1218</v>
+        <v>1101</v>
       </c>
       <c r="O35" t="s">
         <v>610</v>
@@ -21584,28 +21662,28 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1219</v>
-      </c>
-      <c r="B36" t="s">
-        <v>1219</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1039</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1214</v>
-      </c>
-      <c r="E36" t="s">
-        <v>527</v>
-      </c>
-      <c r="F36" t="s">
-        <v>1214</v>
+        <v>1202</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>1208</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>1202</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H36" t="s">
-        <v>1215</v>
+        <v>1203</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>7</v>
@@ -21613,8 +21691,11 @@
       <c r="J36" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="L36" s="6" t="s">
+        <v>1351</v>
+      </c>
       <c r="M36" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
       <c r="O36" t="s">
         <v>610</v>
@@ -21625,28 +21706,28 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>1213</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>1213</v>
+        <v>1219</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1219</v>
       </c>
       <c r="C37" t="s">
-        <v>1204</v>
+        <v>1039</v>
       </c>
       <c r="D37" t="s">
-        <v>1205</v>
+        <v>1214</v>
       </c>
       <c r="E37" t="s">
-        <v>1207</v>
+        <v>527</v>
       </c>
       <c r="F37" t="s">
-        <v>1205</v>
+        <v>1214</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H37" t="s">
-        <v>1209</v>
+        <v>1215</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>7</v>
@@ -21654,8 +21735,11 @@
       <c r="J37" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="L37" s="6" t="s">
+        <v>1365</v>
+      </c>
       <c r="M37" t="s">
-        <v>1211</v>
+        <v>1216</v>
       </c>
       <c r="O37" t="s">
         <v>610</v>
@@ -21675,19 +21759,19 @@
         <v>1204</v>
       </c>
       <c r="D38" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="E38" t="s">
         <v>1207</v>
       </c>
       <c r="F38" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H38" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>7</v>
@@ -21695,8 +21779,11 @@
       <c r="J38" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="L38" s="6" t="s">
+        <v>1354</v>
+      </c>
       <c r="M38" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="O38" t="s">
         <v>610</v>
@@ -21707,40 +21794,43 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B39" t="s">
-        <v>1038</v>
+        <v>1213</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>1213</v>
       </c>
       <c r="C39" t="s">
-        <v>1039</v>
+        <v>1204</v>
       </c>
       <c r="D39" t="s">
-        <v>1040</v>
+        <v>1206</v>
       </c>
       <c r="E39" t="s">
-        <v>751</v>
+        <v>1207</v>
       </c>
       <c r="F39" t="s">
-        <v>1040</v>
-      </c>
-      <c r="G39" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G39" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H39" t="s">
-        <v>1041</v>
-      </c>
-      <c r="I39" t="s">
-        <v>7</v>
-      </c>
-      <c r="J39" t="s">
+        <v>1210</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J39" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="L39" s="6" t="s">
+        <v>1352</v>
+      </c>
       <c r="M39" t="s">
-        <v>1042</v>
+        <v>1212</v>
       </c>
       <c r="O39" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P39" t="s">
         <v>895</v>
@@ -21757,19 +21847,19 @@
         <v>1039</v>
       </c>
       <c r="D40" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="E40" t="s">
         <v>751</v>
       </c>
       <c r="F40" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="G40" t="s">
         <v>48</v>
       </c>
       <c r="H40" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="I40" t="s">
         <v>7</v>
@@ -21777,8 +21867,11 @@
       <c r="J40" t="s">
         <v>16</v>
       </c>
+      <c r="L40" s="6" t="s">
+        <v>1355</v>
+      </c>
       <c r="M40" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="O40" t="s">
         <v>1043</v>
@@ -21798,19 +21891,19 @@
         <v>1039</v>
       </c>
       <c r="D41" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="E41" t="s">
         <v>751</v>
       </c>
       <c r="F41" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="G41" t="s">
         <v>48</v>
       </c>
       <c r="H41" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="I41" t="s">
         <v>7</v>
@@ -21818,8 +21911,11 @@
       <c r="J41" t="s">
         <v>16</v>
       </c>
+      <c r="L41" s="6" t="s">
+        <v>1356</v>
+      </c>
       <c r="M41" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="O41" t="s">
         <v>1043</v>
@@ -21839,19 +21935,19 @@
         <v>1039</v>
       </c>
       <c r="D42" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="E42" t="s">
         <v>751</v>
       </c>
       <c r="F42" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="G42" t="s">
         <v>48</v>
       </c>
       <c r="H42" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="I42" t="s">
         <v>7</v>
@@ -21859,8 +21955,11 @@
       <c r="J42" t="s">
         <v>16</v>
       </c>
+      <c r="L42" s="6" t="s">
+        <v>1357</v>
+      </c>
       <c r="M42" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="O42" t="s">
         <v>1043</v>
@@ -21880,19 +21979,19 @@
         <v>1039</v>
       </c>
       <c r="D43" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="E43" t="s">
         <v>751</v>
       </c>
       <c r="F43" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="G43" t="s">
         <v>48</v>
       </c>
       <c r="H43" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="I43" t="s">
         <v>7</v>
@@ -21900,8 +21999,11 @@
       <c r="J43" t="s">
         <v>16</v>
       </c>
+      <c r="L43" s="6" t="s">
+        <v>1358</v>
+      </c>
       <c r="M43" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="O43" t="s">
         <v>1043</v>
@@ -21921,19 +22023,19 @@
         <v>1039</v>
       </c>
       <c r="D44" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="E44" t="s">
         <v>751</v>
       </c>
       <c r="F44" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="G44" t="s">
         <v>48</v>
       </c>
       <c r="H44" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="I44" t="s">
         <v>7</v>
@@ -21941,8 +22043,11 @@
       <c r="J44" t="s">
         <v>16</v>
       </c>
+      <c r="L44" s="6" t="s">
+        <v>1359</v>
+      </c>
       <c r="M44" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
       <c r="O44" t="s">
         <v>1043</v>
@@ -21962,19 +22067,19 @@
         <v>1039</v>
       </c>
       <c r="D45" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="E45" t="s">
         <v>751</v>
       </c>
       <c r="F45" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="G45" t="s">
         <v>48</v>
       </c>
       <c r="H45" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="I45" t="s">
         <v>7</v>
@@ -21982,8 +22087,11 @@
       <c r="J45" t="s">
         <v>16</v>
       </c>
+      <c r="L45" s="6" t="s">
+        <v>1360</v>
+      </c>
       <c r="M45" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="O45" t="s">
         <v>1043</v>
@@ -22003,19 +22111,19 @@
         <v>1039</v>
       </c>
       <c r="D46" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="E46" t="s">
         <v>751</v>
       </c>
       <c r="F46" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="G46" t="s">
         <v>48</v>
       </c>
       <c r="H46" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="I46" t="s">
         <v>7</v>
@@ -22023,8 +22131,11 @@
       <c r="J46" t="s">
         <v>16</v>
       </c>
+      <c r="L46" s="6" t="s">
+        <v>1361</v>
+      </c>
       <c r="M46" t="s">
-        <v>1064</v>
+        <v>1061</v>
       </c>
       <c r="O46" t="s">
         <v>1043</v>
@@ -22044,19 +22155,19 @@
         <v>1039</v>
       </c>
       <c r="D47" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="E47" t="s">
         <v>751</v>
       </c>
       <c r="F47" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="G47" t="s">
         <v>48</v>
       </c>
       <c r="H47" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="I47" t="s">
         <v>7</v>
@@ -22064,8 +22175,11 @@
       <c r="J47" t="s">
         <v>16</v>
       </c>
+      <c r="L47" s="6" t="s">
+        <v>1362</v>
+      </c>
       <c r="M47" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
       <c r="O47" t="s">
         <v>1043</v>
@@ -22085,19 +22199,19 @@
         <v>1039</v>
       </c>
       <c r="D48" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E48" t="s">
         <v>751</v>
       </c>
       <c r="F48" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="G48" t="s">
         <v>48</v>
       </c>
       <c r="H48" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="I48" t="s">
         <v>7</v>
@@ -22105,8 +22219,11 @@
       <c r="J48" t="s">
         <v>16</v>
       </c>
+      <c r="L48" s="6" t="s">
+        <v>1363</v>
+      </c>
       <c r="M48" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="O48" t="s">
         <v>1043</v>
@@ -22117,28 +22234,28 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>611</v>
+        <v>1037</v>
       </c>
       <c r="B49" t="s">
-        <v>611</v>
+        <v>1038</v>
       </c>
       <c r="C49" t="s">
-        <v>617</v>
+        <v>1039</v>
       </c>
       <c r="D49" t="s">
-        <v>611</v>
+        <v>1068</v>
       </c>
       <c r="E49" t="s">
-        <v>525</v>
+        <v>751</v>
       </c>
       <c r="F49" t="s">
-        <v>611</v>
+        <v>1068</v>
       </c>
       <c r="G49" t="s">
         <v>48</v>
       </c>
       <c r="H49" t="s">
-        <v>616</v>
+        <v>1069</v>
       </c>
       <c r="I49" t="s">
         <v>7</v>
@@ -22146,40 +22263,43 @@
       <c r="J49" t="s">
         <v>16</v>
       </c>
+      <c r="L49" s="6" t="s">
+        <v>1364</v>
+      </c>
       <c r="M49" t="s">
-        <v>878</v>
+        <v>1070</v>
       </c>
       <c r="O49" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P49" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>875</v>
+        <v>611</v>
       </c>
       <c r="B50" t="s">
-        <v>875</v>
+        <v>611</v>
       </c>
       <c r="C50" t="s">
-        <v>877</v>
+        <v>617</v>
       </c>
       <c r="D50" t="s">
-        <v>874</v>
+        <v>611</v>
       </c>
       <c r="E50" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="F50" t="s">
-        <v>874</v>
+        <v>611</v>
       </c>
       <c r="G50" t="s">
         <v>48</v>
       </c>
       <c r="H50" t="s">
-        <v>876</v>
+        <v>616</v>
       </c>
       <c r="I50" t="s">
         <v>7</v>
@@ -22188,39 +22308,39 @@
         <v>16</v>
       </c>
       <c r="M50" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="O50" t="s">
         <v>618</v>
       </c>
       <c r="P50" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>887</v>
+        <v>875</v>
       </c>
       <c r="B51" t="s">
-        <v>886</v>
+        <v>875</v>
       </c>
       <c r="C51" t="s">
-        <v>886</v>
+        <v>877</v>
       </c>
       <c r="D51" t="s">
-        <v>880</v>
+        <v>874</v>
       </c>
       <c r="E51" t="s">
         <v>527</v>
       </c>
       <c r="F51" t="s">
-        <v>880</v>
+        <v>874</v>
       </c>
       <c r="G51" t="s">
         <v>48</v>
       </c>
       <c r="H51" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="I51" t="s">
         <v>7</v>
@@ -22229,7 +22349,7 @@
         <v>16</v>
       </c>
       <c r="M51" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="O51" t="s">
         <v>618</v>
@@ -22240,7 +22360,7 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B52" t="s">
         <v>886</v>
@@ -22249,19 +22369,19 @@
         <v>886</v>
       </c>
       <c r="D52" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="E52" t="s">
         <v>527</v>
       </c>
       <c r="F52" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="G52" t="s">
         <v>48</v>
       </c>
       <c r="H52" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="I52" t="s">
         <v>7</v>
@@ -22270,7 +22390,7 @@
         <v>16</v>
       </c>
       <c r="M52" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="O52" t="s">
         <v>618</v>
@@ -22281,28 +22401,28 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>861</v>
+        <v>888</v>
       </c>
       <c r="B53" t="s">
-        <v>861</v>
+        <v>886</v>
       </c>
       <c r="C53" t="s">
-        <v>862</v>
+        <v>886</v>
       </c>
       <c r="D53" t="s">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="E53" t="s">
-        <v>864</v>
+        <v>527</v>
       </c>
       <c r="F53" t="s">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="G53" t="s">
         <v>48</v>
       </c>
       <c r="H53" t="s">
-        <v>865</v>
+        <v>884</v>
       </c>
       <c r="I53" t="s">
         <v>7</v>
@@ -22311,10 +22431,10 @@
         <v>16</v>
       </c>
       <c r="M53" t="s">
-        <v>866</v>
+        <v>885</v>
       </c>
       <c r="O53" t="s">
-        <v>867</v>
+        <v>618</v>
       </c>
       <c r="P53" t="s">
         <v>895</v>
@@ -22322,40 +22442,40 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>930</v>
+        <v>861</v>
       </c>
       <c r="B54" t="s">
-        <v>615</v>
+        <v>861</v>
       </c>
       <c r="C54" t="s">
-        <v>615</v>
+        <v>862</v>
       </c>
       <c r="D54" t="s">
-        <v>931</v>
+        <v>863</v>
       </c>
       <c r="E54" t="s">
-        <v>527</v>
+        <v>864</v>
       </c>
       <c r="F54" t="s">
-        <v>931</v>
+        <v>863</v>
       </c>
       <c r="G54" t="s">
         <v>48</v>
       </c>
       <c r="H54" t="s">
-        <v>932</v>
+        <v>865</v>
       </c>
       <c r="I54" t="s">
         <v>7</v>
       </c>
       <c r="J54" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M54" t="s">
-        <v>934</v>
+        <v>866</v>
       </c>
       <c r="O54" t="s">
-        <v>933</v>
+        <v>867</v>
       </c>
       <c r="P54" t="s">
         <v>895</v>
@@ -22363,40 +22483,40 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>1111</v>
+        <v>930</v>
       </c>
       <c r="B55" t="s">
-        <v>1111</v>
+        <v>615</v>
       </c>
       <c r="C55" t="s">
-        <v>1110</v>
+        <v>615</v>
       </c>
       <c r="D55" t="s">
-        <v>1112</v>
+        <v>931</v>
       </c>
       <c r="E55" t="s">
-        <v>1106</v>
+        <v>527</v>
       </c>
       <c r="F55" t="s">
-        <v>1116</v>
+        <v>931</v>
       </c>
       <c r="G55" t="s">
         <v>48</v>
       </c>
       <c r="H55" t="s">
-        <v>1120</v>
+        <v>932</v>
       </c>
       <c r="I55" t="s">
         <v>7</v>
       </c>
       <c r="J55" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M55" t="s">
-        <v>1109</v>
+        <v>934</v>
       </c>
       <c r="O55" t="s">
-        <v>565</v>
+        <v>933</v>
       </c>
       <c r="P55" t="s">
         <v>895</v>
@@ -22413,19 +22533,19 @@
         <v>1110</v>
       </c>
       <c r="D56" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="E56" t="s">
         <v>1106</v>
       </c>
       <c r="F56" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="G56" t="s">
         <v>48</v>
       </c>
       <c r="H56" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="I56" t="s">
         <v>7</v>
@@ -22454,19 +22574,19 @@
         <v>1110</v>
       </c>
       <c r="D57" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="E57" t="s">
         <v>1106</v>
       </c>
       <c r="F57" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="G57" t="s">
         <v>48</v>
       </c>
       <c r="H57" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="I57" t="s">
         <v>7</v>
@@ -22495,19 +22615,19 @@
         <v>1110</v>
       </c>
       <c r="D58" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="E58" t="s">
         <v>1106</v>
       </c>
       <c r="F58" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="G58" t="s">
         <v>48</v>
       </c>
       <c r="H58" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="I58" t="s">
         <v>7</v>
@@ -22536,19 +22656,19 @@
         <v>1110</v>
       </c>
       <c r="D59" t="s">
-        <v>1105</v>
+        <v>1115</v>
       </c>
       <c r="E59" t="s">
         <v>1106</v>
       </c>
       <c r="F59" t="s">
-        <v>1107</v>
+        <v>1119</v>
       </c>
       <c r="G59" t="s">
         <v>48</v>
       </c>
       <c r="H59" t="s">
-        <v>1108</v>
+        <v>1123</v>
       </c>
       <c r="I59" t="s">
         <v>7</v>
@@ -22568,28 +22688,28 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>556</v>
+        <v>1111</v>
       </c>
       <c r="B60" t="s">
-        <v>562</v>
+        <v>1111</v>
       </c>
       <c r="C60" t="s">
-        <v>562</v>
+        <v>1110</v>
       </c>
       <c r="D60" t="s">
-        <v>556</v>
+        <v>1105</v>
       </c>
       <c r="E60" t="s">
-        <v>557</v>
+        <v>1106</v>
       </c>
       <c r="F60" t="s">
-        <v>556</v>
+        <v>1107</v>
       </c>
       <c r="G60" t="s">
-        <v>558</v>
+        <v>48</v>
       </c>
       <c r="H60" t="s">
-        <v>561</v>
+        <v>1108</v>
       </c>
       <c r="I60" t="s">
         <v>7</v>
@@ -22598,39 +22718,39 @@
         <v>16</v>
       </c>
       <c r="M60" t="s">
-        <v>566</v>
+        <v>1109</v>
       </c>
       <c r="O60" t="s">
         <v>565</v>
       </c>
       <c r="P60" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="B61" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C61" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D61" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="E61" t="s">
         <v>557</v>
       </c>
       <c r="F61" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="G61" t="s">
-        <v>48</v>
+        <v>558</v>
       </c>
       <c r="H61" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="I61" t="s">
         <v>7</v>
@@ -22639,7 +22759,7 @@
         <v>16</v>
       </c>
       <c r="M61" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="O61" t="s">
         <v>565</v>
@@ -22650,28 +22770,28 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>1246</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>1246</v>
+        <v>559</v>
+      </c>
+      <c r="B62" t="s">
+        <v>564</v>
       </c>
       <c r="C62" t="s">
-        <v>1248</v>
+        <v>564</v>
       </c>
       <c r="D62" t="s">
-        <v>1244</v>
+        <v>559</v>
       </c>
       <c r="E62" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="F62" t="s">
-        <v>1244</v>
+        <v>559</v>
       </c>
       <c r="G62" t="s">
         <v>48</v>
       </c>
       <c r="H62" t="s">
-        <v>1245</v>
+        <v>560</v>
       </c>
       <c r="I62" t="s">
         <v>7</v>
@@ -22680,12 +22800,53 @@
         <v>16</v>
       </c>
       <c r="M62" t="s">
+        <v>567</v>
+      </c>
+      <c r="O62" t="s">
+        <v>565</v>
+      </c>
+      <c r="P62" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1244</v>
+      </c>
+      <c r="E63" t="s">
+        <v>527</v>
+      </c>
+      <c r="F63" t="s">
+        <v>1244</v>
+      </c>
+      <c r="G63" t="s">
+        <v>48</v>
+      </c>
+      <c r="H63" t="s">
+        <v>1245</v>
+      </c>
+      <c r="I63" t="s">
+        <v>7</v>
+      </c>
+      <c r="J63" t="s">
+        <v>16</v>
+      </c>
+      <c r="M63" t="s">
         <v>1247</v>
       </c>
-      <c r="O62" t="s">
+      <c r="O63" t="s">
         <v>1243</v>
       </c>
-      <c r="P62" t="s">
+      <c r="P63" t="s">
         <v>895</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix bad info for RP235xx
</commit_message>
<xml_diff>
--- a/Moonlight_Library.xlsx
+++ b/Moonlight_Library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mani\Documents\Projects\altium\libraries\Moonlight_Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6551DF-3A19-4A3F-8774-F2A28783B9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B9F30E-F43B-4C37-A6F0-FFE2A76D98CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="905" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5847" uniqueCount="1366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5851" uniqueCount="1370">
   <si>
     <t>Symbol Ref</t>
   </si>
@@ -4148,6 +4148,18 @@
   </si>
   <si>
     <t>0.6-34.2V</t>
+  </si>
+  <si>
+    <t>2648-SC1509-A4CT-ND</t>
+  </si>
+  <si>
+    <t>2648-SC1511-A4CT-ND</t>
+  </si>
+  <si>
+    <t>2648-SC1510-A4CT-ND</t>
+  </si>
+  <si>
+    <t>2648-SC1512-A4CT-ND</t>
   </si>
 </sst>
 </file>
@@ -20309,7 +20321,7 @@
         <v>1343</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1345</v>
+        <v>1337</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
@@ -20319,6 +20331,9 @@
       </c>
       <c r="G3" t="s">
         <v>48</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>1366</v>
       </c>
       <c r="I3" t="s">
         <v>7</v>
@@ -20347,7 +20362,7 @@
         <v>1343</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1345</v>
+        <v>1338</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -20357,6 +20372,9 @@
       </c>
       <c r="G4" t="s">
         <v>48</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>1367</v>
       </c>
       <c r="I4" t="s">
         <v>7</v>
@@ -20385,7 +20403,7 @@
         <v>1344</v>
       </c>
       <c r="D5" t="s">
-        <v>1336</v>
+        <v>1339</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
@@ -20395,6 +20413,9 @@
       </c>
       <c r="G5" t="s">
         <v>48</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1368</v>
       </c>
       <c r="I5" t="s">
         <v>7</v>
@@ -20423,7 +20444,7 @@
         <v>1344</v>
       </c>
       <c r="D6" t="s">
-        <v>1336</v>
+        <v>1340</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
@@ -20433,6 +20454,9 @@
       </c>
       <c r="G6" t="s">
         <v>48</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1369</v>
       </c>
       <c r="I6" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Add FRAM IC, rename Flash directory to Memory and remove reference to voltage spec from XC6222 regulator name
</commit_message>
<xml_diff>
--- a/Moonlight_Library.xlsx
+++ b/Moonlight_Library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mani\Documents\Projects\altium\libraries\Moonlight_Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B9F30E-F43B-4C37-A6F0-FFE2A76D98CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBE0CCC-4198-4154-AB69-AB7970E6EF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="905" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5851" uniqueCount="1370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5864" uniqueCount="1377">
   <si>
     <t>Symbol Ref</t>
   </si>
@@ -4160,6 +4160,27 @@
   </si>
   <si>
     <t>2648-SC1512-A4CT-ND</t>
+  </si>
+  <si>
+    <t>CY15B016Q</t>
+  </si>
+  <si>
+    <t>Infineon Technologies</t>
+  </si>
+  <si>
+    <t>CY15B016Q-SXET</t>
+  </si>
+  <si>
+    <t>448-CY15B016Q-SXETCT-ND</t>
+  </si>
+  <si>
+    <t>16 Kbit SPI FRAM memory</t>
+  </si>
+  <si>
+    <t>FRAM Memory</t>
+  </si>
+  <si>
+    <t>XC6222</t>
   </si>
 </sst>
 </file>
@@ -20199,7 +20220,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B93A8C-0336-4B42-880D-67109C66C120}">
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" style="6" bestFit="1" customWidth="1"/>
@@ -20719,28 +20740,28 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>514</v>
+        <v>1370</v>
       </c>
       <c r="B13" t="s">
-        <v>514</v>
+        <v>584</v>
       </c>
       <c r="C13" t="s">
-        <v>539</v>
+        <v>584</v>
       </c>
       <c r="D13" t="s">
-        <v>514</v>
+        <v>1370</v>
       </c>
       <c r="E13" t="s">
-        <v>524</v>
+        <v>1371</v>
       </c>
       <c r="F13" t="s">
-        <v>514</v>
+        <v>1372</v>
       </c>
       <c r="G13" t="s">
         <v>48</v>
       </c>
-      <c r="H13" t="s">
-        <v>530</v>
+      <c r="H13" s="4" t="s">
+        <v>1373</v>
       </c>
       <c r="I13" t="s">
         <v>7</v>
@@ -20749,10 +20770,10 @@
         <v>16</v>
       </c>
       <c r="M13" t="s">
-        <v>554</v>
+        <v>1374</v>
       </c>
       <c r="O13" t="s">
-        <v>521</v>
+        <v>1375</v>
       </c>
       <c r="P13" t="s">
         <v>895</v>
@@ -20760,28 +20781,28 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B14" t="s">
-        <v>549</v>
+        <v>514</v>
       </c>
       <c r="C14" t="s">
-        <v>531</v>
+        <v>539</v>
       </c>
       <c r="D14" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E14" t="s">
         <v>524</v>
       </c>
       <c r="F14" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="G14" t="s">
         <v>48</v>
       </c>
       <c r="H14" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="I14" t="s">
         <v>7</v>
@@ -20790,21 +20811,18 @@
         <v>16</v>
       </c>
       <c r="M14" t="s">
-        <v>553</v>
-      </c>
-      <c r="N14" t="s">
-        <v>414</v>
+        <v>554</v>
       </c>
       <c r="O14" t="s">
         <v>521</v>
       </c>
       <c r="P14" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>547</v>
+        <v>515</v>
       </c>
       <c r="B15" t="s">
         <v>549</v>
@@ -20813,19 +20831,19 @@
         <v>531</v>
       </c>
       <c r="D15" t="s">
-        <v>547</v>
+        <v>515</v>
       </c>
       <c r="E15" t="s">
         <v>524</v>
       </c>
       <c r="F15" t="s">
-        <v>547</v>
+        <v>515</v>
       </c>
       <c r="G15" t="s">
         <v>48</v>
       </c>
       <c r="H15" t="s">
-        <v>550</v>
+        <v>533</v>
       </c>
       <c r="I15" t="s">
         <v>7</v>
@@ -20836,6 +20854,9 @@
       <c r="M15" t="s">
         <v>553</v>
       </c>
+      <c r="N15" t="s">
+        <v>414</v>
+      </c>
       <c r="O15" t="s">
         <v>521</v>
       </c>
@@ -20845,28 +20866,28 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B16" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C16" t="s">
-        <v>555</v>
+        <v>531</v>
       </c>
       <c r="D16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E16" t="s">
         <v>524</v>
       </c>
       <c r="F16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G16" t="s">
         <v>48</v>
       </c>
       <c r="H16" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I16" t="s">
         <v>7</v>
@@ -20875,39 +20896,39 @@
         <v>16</v>
       </c>
       <c r="M16" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="O16" t="s">
         <v>521</v>
       </c>
       <c r="P16" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="B17" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="C17" t="s">
-        <v>534</v>
+        <v>555</v>
       </c>
       <c r="D17" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="E17" t="s">
         <v>524</v>
       </c>
       <c r="F17" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="G17" t="s">
         <v>48</v>
       </c>
       <c r="H17" t="s">
-        <v>535</v>
+        <v>551</v>
       </c>
       <c r="I17" t="s">
         <v>7</v>
@@ -20916,39 +20937,39 @@
         <v>16</v>
       </c>
       <c r="M17" t="s">
-        <v>543</v>
+        <v>552</v>
       </c>
       <c r="O17" t="s">
         <v>521</v>
       </c>
       <c r="P17" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B18" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C18" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D18" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E18" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F18" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="G18" t="s">
         <v>48</v>
       </c>
       <c r="H18" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="I18" t="s">
         <v>7</v>
@@ -20957,7 +20978,7 @@
         <v>16</v>
       </c>
       <c r="M18" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="O18" t="s">
         <v>521</v>
@@ -20968,28 +20989,28 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B19" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C19" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="D19" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E19" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F19" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="G19" t="s">
         <v>48</v>
       </c>
       <c r="H19" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="I19" t="s">
         <v>7</v>
@@ -21009,28 +21030,28 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="B20" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="C20" t="s">
-        <v>532</v>
+        <v>540</v>
       </c>
       <c r="D20" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="E20" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="F20" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="G20" t="s">
         <v>48</v>
       </c>
       <c r="H20" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="I20" t="s">
         <v>7</v>
@@ -21039,7 +21060,7 @@
         <v>16</v>
       </c>
       <c r="M20" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="O20" t="s">
         <v>521</v>
@@ -21050,28 +21071,28 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B21" t="s">
-        <v>542</v>
+        <v>523</v>
       </c>
       <c r="C21" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="D21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E21" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G21" t="s">
         <v>48</v>
       </c>
       <c r="H21" t="s">
-        <v>541</v>
+        <v>529</v>
       </c>
       <c r="I21" t="s">
         <v>7</v>
@@ -21080,7 +21101,7 @@
         <v>16</v>
       </c>
       <c r="M21" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="O21" t="s">
         <v>521</v>
@@ -21091,28 +21112,28 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>854</v>
+        <v>522</v>
       </c>
       <c r="B22" t="s">
-        <v>855</v>
+        <v>542</v>
       </c>
       <c r="C22" t="s">
-        <v>855</v>
+        <v>542</v>
       </c>
       <c r="D22" t="s">
-        <v>856</v>
+        <v>522</v>
       </c>
       <c r="E22" t="s">
-        <v>857</v>
+        <v>527</v>
       </c>
       <c r="F22" t="s">
-        <v>856</v>
+        <v>522</v>
       </c>
       <c r="G22" t="s">
-        <v>858</v>
+        <v>48</v>
       </c>
       <c r="H22" t="s">
-        <v>859</v>
+        <v>541</v>
       </c>
       <c r="I22" t="s">
         <v>7</v>
@@ -21121,39 +21142,39 @@
         <v>16</v>
       </c>
       <c r="M22" t="s">
-        <v>860</v>
+        <v>545</v>
       </c>
       <c r="O22" t="s">
         <v>521</v>
       </c>
       <c r="P22" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>1034</v>
+        <v>854</v>
       </c>
       <c r="B23" t="s">
-        <v>1034</v>
+        <v>855</v>
       </c>
       <c r="C23" t="s">
-        <v>1034</v>
+        <v>855</v>
       </c>
       <c r="D23" t="s">
-        <v>1034</v>
+        <v>856</v>
       </c>
       <c r="E23" t="s">
-        <v>527</v>
+        <v>857</v>
       </c>
       <c r="F23" t="s">
-        <v>1034</v>
+        <v>856</v>
       </c>
       <c r="G23" t="s">
-        <v>48</v>
+        <v>858</v>
       </c>
       <c r="H23" t="s">
-        <v>1035</v>
+        <v>859</v>
       </c>
       <c r="I23" t="s">
         <v>7</v>
@@ -21162,10 +21183,7 @@
         <v>16</v>
       </c>
       <c r="M23" t="s">
-        <v>1036</v>
-      </c>
-      <c r="N23" t="s">
-        <v>414</v>
+        <v>860</v>
       </c>
       <c r="O23" t="s">
         <v>521</v>
@@ -21176,28 +21194,28 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>588</v>
+        <v>1034</v>
       </c>
       <c r="B24" t="s">
-        <v>584</v>
+        <v>1034</v>
       </c>
       <c r="C24" t="s">
-        <v>584</v>
+        <v>1034</v>
       </c>
       <c r="D24" t="s">
-        <v>589</v>
+        <v>1034</v>
       </c>
       <c r="E24" t="s">
         <v>527</v>
       </c>
       <c r="F24" t="s">
-        <v>589</v>
+        <v>1034</v>
       </c>
       <c r="G24" t="s">
         <v>48</v>
       </c>
       <c r="H24" t="s">
-        <v>590</v>
+        <v>1035</v>
       </c>
       <c r="I24" t="s">
         <v>7</v>
@@ -21206,39 +21224,42 @@
         <v>16</v>
       </c>
       <c r="M24" t="s">
-        <v>599</v>
+        <v>1036</v>
+      </c>
+      <c r="N24" t="s">
+        <v>414</v>
       </c>
       <c r="O24" t="s">
-        <v>597</v>
+        <v>521</v>
       </c>
       <c r="P24" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="B25" t="s">
-        <v>602</v>
+        <v>584</v>
       </c>
       <c r="C25" t="s">
-        <v>603</v>
+        <v>584</v>
       </c>
       <c r="D25" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="E25" t="s">
-        <v>594</v>
+        <v>527</v>
       </c>
       <c r="F25" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="G25" t="s">
         <v>48</v>
       </c>
       <c r="H25" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="I25" t="s">
         <v>7</v>
@@ -21247,7 +21268,7 @@
         <v>16</v>
       </c>
       <c r="M25" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="O25" t="s">
         <v>597</v>
@@ -21258,28 +21279,28 @@
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="B26" t="s">
-        <v>584</v>
+        <v>602</v>
       </c>
       <c r="C26" t="s">
-        <v>584</v>
+        <v>603</v>
       </c>
       <c r="D26" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="E26" t="s">
-        <v>527</v>
+        <v>594</v>
       </c>
       <c r="F26" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="G26" t="s">
         <v>48</v>
       </c>
       <c r="H26" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="I26" t="s">
         <v>7</v>
@@ -21288,39 +21309,39 @@
         <v>16</v>
       </c>
       <c r="M26" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="O26" t="s">
         <v>597</v>
       </c>
       <c r="P26" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>1253</v>
+        <v>601</v>
       </c>
       <c r="B27" t="s">
-        <v>1255</v>
+        <v>584</v>
       </c>
       <c r="C27" t="s">
-        <v>1254</v>
+        <v>584</v>
       </c>
       <c r="D27" t="s">
-        <v>1255</v>
+        <v>595</v>
       </c>
       <c r="E27" t="s">
-        <v>1207</v>
+        <v>527</v>
       </c>
       <c r="F27" t="s">
-        <v>1255</v>
+        <v>595</v>
       </c>
       <c r="G27" t="s">
         <v>48</v>
       </c>
       <c r="H27" t="s">
-        <v>1256</v>
+        <v>596</v>
       </c>
       <c r="I27" t="s">
         <v>7</v>
@@ -21329,7 +21350,7 @@
         <v>16</v>
       </c>
       <c r="M27" t="s">
-        <v>1257</v>
+        <v>600</v>
       </c>
       <c r="O27" t="s">
         <v>597</v>
@@ -21340,28 +21361,28 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>1275</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>1275</v>
+        <v>1253</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1255</v>
       </c>
       <c r="C28" t="s">
-        <v>1276</v>
+        <v>1254</v>
       </c>
       <c r="D28" t="s">
-        <v>1277</v>
+        <v>1255</v>
       </c>
       <c r="E28" t="s">
         <v>1207</v>
       </c>
       <c r="F28" t="s">
-        <v>1277</v>
+        <v>1255</v>
       </c>
       <c r="G28" t="s">
         <v>48</v>
       </c>
       <c r="H28" t="s">
-        <v>1278</v>
+        <v>1256</v>
       </c>
       <c r="I28" t="s">
         <v>7</v>
@@ -21370,10 +21391,10 @@
         <v>16</v>
       </c>
       <c r="M28" t="s">
-        <v>1279</v>
+        <v>1257</v>
       </c>
       <c r="O28" t="s">
-        <v>1274</v>
+        <v>597</v>
       </c>
       <c r="P28" t="s">
         <v>895</v>
@@ -21381,28 +21402,28 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>868</v>
-      </c>
-      <c r="B29" t="s">
-        <v>869</v>
+        <v>1275</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>1275</v>
       </c>
       <c r="C29" t="s">
-        <v>869</v>
+        <v>1276</v>
       </c>
       <c r="D29" t="s">
-        <v>870</v>
+        <v>1277</v>
       </c>
       <c r="E29" t="s">
-        <v>751</v>
+        <v>1207</v>
       </c>
       <c r="F29" t="s">
-        <v>870</v>
+        <v>1277</v>
       </c>
       <c r="G29" t="s">
         <v>48</v>
       </c>
       <c r="H29" t="s">
-        <v>871</v>
+        <v>1278</v>
       </c>
       <c r="I29" t="s">
         <v>7</v>
@@ -21411,10 +21432,10 @@
         <v>16</v>
       </c>
       <c r="M29" t="s">
-        <v>873</v>
+        <v>1279</v>
       </c>
       <c r="O29" t="s">
-        <v>872</v>
+        <v>1274</v>
       </c>
       <c r="P29" t="s">
         <v>895</v>
@@ -21422,28 +21443,28 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>606</v>
+        <v>868</v>
       </c>
       <c r="B30" t="s">
-        <v>609</v>
+        <v>869</v>
       </c>
       <c r="C30" t="s">
-        <v>609</v>
+        <v>869</v>
       </c>
       <c r="D30" t="s">
-        <v>606</v>
+        <v>870</v>
       </c>
       <c r="E30" t="s">
-        <v>608</v>
+        <v>751</v>
       </c>
       <c r="F30" t="s">
-        <v>606</v>
+        <v>870</v>
       </c>
       <c r="G30" t="s">
         <v>48</v>
       </c>
       <c r="H30" t="s">
-        <v>607</v>
+        <v>871</v>
       </c>
       <c r="I30" t="s">
         <v>7</v>
@@ -21451,43 +21472,40 @@
       <c r="J30" t="s">
         <v>16</v>
       </c>
-      <c r="L30" t="s">
-        <v>1349</v>
-      </c>
       <c r="M30" t="s">
-        <v>1217</v>
+        <v>873</v>
       </c>
       <c r="O30" t="s">
-        <v>610</v>
+        <v>872</v>
       </c>
       <c r="P30" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="B31" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="C31" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="D31" t="s">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="E31" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="F31" t="s">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="G31" t="s">
         <v>48</v>
       </c>
       <c r="H31" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="I31" t="s">
         <v>7</v>
@@ -21496,21 +21514,21 @@
         <v>16</v>
       </c>
       <c r="L31" t="s">
-        <v>1352</v>
+        <v>1349</v>
       </c>
       <c r="M31" t="s">
-        <v>1022</v>
+        <v>1217</v>
       </c>
       <c r="O31" t="s">
         <v>610</v>
       </c>
       <c r="P31" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1348</v>
+        <v>1376</v>
       </c>
       <c r="B32" t="s">
         <v>615</v>
@@ -21519,19 +21537,19 @@
         <v>615</v>
       </c>
       <c r="D32" t="s">
-        <v>1348</v>
+        <v>613</v>
       </c>
       <c r="E32" t="s">
         <v>614</v>
       </c>
       <c r="F32" t="s">
-        <v>1348</v>
+        <v>613</v>
       </c>
       <c r="G32" t="s">
         <v>48</v>
       </c>
       <c r="H32" t="s">
-        <v>1347</v>
+        <v>612</v>
       </c>
       <c r="I32" t="s">
         <v>7</v>
@@ -21540,42 +21558,42 @@
         <v>16</v>
       </c>
       <c r="L32" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="M32" t="s">
-        <v>1346</v>
+        <v>1022</v>
       </c>
       <c r="O32" t="s">
         <v>610</v>
       </c>
       <c r="P32" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>1019</v>
+        <v>1376</v>
       </c>
       <c r="B33" t="s">
-        <v>718</v>
+        <v>615</v>
       </c>
       <c r="C33" t="s">
-        <v>718</v>
+        <v>615</v>
       </c>
       <c r="D33" t="s">
-        <v>1019</v>
+        <v>1348</v>
       </c>
       <c r="E33" t="s">
-        <v>719</v>
+        <v>614</v>
       </c>
       <c r="F33" t="s">
-        <v>1019</v>
+        <v>1348</v>
       </c>
       <c r="G33" t="s">
         <v>48</v>
       </c>
       <c r="H33" t="s">
-        <v>1020</v>
+        <v>1347</v>
       </c>
       <c r="I33" t="s">
         <v>7</v>
@@ -21584,54 +21602,54 @@
         <v>16</v>
       </c>
       <c r="L33" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="M33" t="s">
-        <v>1021</v>
+        <v>1346</v>
       </c>
       <c r="O33" t="s">
         <v>610</v>
       </c>
       <c r="P33" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="6">
-        <v>7805</v>
+      <c r="A34" s="6" t="s">
+        <v>1019</v>
       </c>
       <c r="B34" t="s">
-        <v>1079</v>
+        <v>718</v>
       </c>
       <c r="C34" t="s">
-        <v>1079</v>
+        <v>718</v>
       </c>
       <c r="D34" t="s">
-        <v>1080</v>
+        <v>1019</v>
       </c>
       <c r="E34" t="s">
-        <v>703</v>
+        <v>719</v>
       </c>
       <c r="F34" t="s">
-        <v>1080</v>
+        <v>1019</v>
       </c>
       <c r="G34" t="s">
         <v>48</v>
       </c>
       <c r="H34" t="s">
-        <v>1081</v>
+        <v>1020</v>
       </c>
       <c r="I34" t="s">
         <v>7</v>
       </c>
       <c r="J34" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L34" t="s">
-        <v>1349</v>
+        <v>1352</v>
       </c>
       <c r="M34" t="s">
-        <v>1082</v>
+        <v>1021</v>
       </c>
       <c r="O34" t="s">
         <v>610</v>
@@ -21641,29 +21659,29 @@
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>1097</v>
+      <c r="A35" s="6">
+        <v>7805</v>
       </c>
       <c r="B35" t="s">
-        <v>1098</v>
+        <v>1079</v>
       </c>
       <c r="C35" t="s">
-        <v>1098</v>
+        <v>1079</v>
       </c>
       <c r="D35" t="s">
-        <v>1099</v>
+        <v>1080</v>
       </c>
       <c r="E35" t="s">
-        <v>525</v>
+        <v>703</v>
       </c>
       <c r="F35" t="s">
-        <v>1099</v>
+        <v>1080</v>
       </c>
       <c r="G35" t="s">
         <v>48</v>
       </c>
       <c r="H35" t="s">
-        <v>1100</v>
+        <v>1081</v>
       </c>
       <c r="I35" t="s">
         <v>7</v>
@@ -21672,10 +21690,10 @@
         <v>8</v>
       </c>
       <c r="L35" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="M35" t="s">
-        <v>1101</v>
+        <v>1082</v>
       </c>
       <c r="O35" t="s">
         <v>610</v>
@@ -21686,40 +21704,40 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>1208</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>1202</v>
-      </c>
-      <c r="G36" s="6" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E36" t="s">
+        <v>525</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G36" t="s">
         <v>48</v>
       </c>
       <c r="H36" t="s">
-        <v>1203</v>
-      </c>
-      <c r="I36" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>1351</v>
+        <v>1100</v>
+      </c>
+      <c r="I36" t="s">
+        <v>7</v>
+      </c>
+      <c r="J36" t="s">
+        <v>8</v>
+      </c>
+      <c r="L36" t="s">
+        <v>1350</v>
       </c>
       <c r="M36" t="s">
-        <v>1218</v>
+        <v>1101</v>
       </c>
       <c r="O36" t="s">
         <v>610</v>
@@ -21730,28 +21748,28 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>1219</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1219</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1039</v>
-      </c>
-      <c r="D37" t="s">
-        <v>1214</v>
-      </c>
-      <c r="E37" t="s">
-        <v>527</v>
-      </c>
-      <c r="F37" t="s">
-        <v>1214</v>
+        <v>1202</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>1208</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>1202</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H37" t="s">
-        <v>1215</v>
+        <v>1203</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>7</v>
@@ -21760,10 +21778,10 @@
         <v>16</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>1365</v>
+        <v>1351</v>
       </c>
       <c r="M37" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
       <c r="O37" t="s">
         <v>610</v>
@@ -21774,28 +21792,28 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>1213</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>1213</v>
+        <v>1219</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1219</v>
       </c>
       <c r="C38" t="s">
-        <v>1204</v>
+        <v>1039</v>
       </c>
       <c r="D38" t="s">
-        <v>1205</v>
+        <v>1214</v>
       </c>
       <c r="E38" t="s">
-        <v>1207</v>
+        <v>527</v>
       </c>
       <c r="F38" t="s">
-        <v>1205</v>
+        <v>1214</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H38" t="s">
-        <v>1209</v>
+        <v>1215</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>7</v>
@@ -21804,10 +21822,10 @@
         <v>16</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>1354</v>
+        <v>1365</v>
       </c>
       <c r="M38" t="s">
-        <v>1211</v>
+        <v>1216</v>
       </c>
       <c r="O38" t="s">
         <v>610</v>
@@ -21827,19 +21845,19 @@
         <v>1204</v>
       </c>
       <c r="D39" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="E39" t="s">
         <v>1207</v>
       </c>
       <c r="F39" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H39" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="I39" s="6" t="s">
         <v>7</v>
@@ -21848,10 +21866,10 @@
         <v>16</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="M39" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="O39" t="s">
         <v>610</v>
@@ -21862,43 +21880,43 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B40" t="s">
-        <v>1038</v>
+        <v>1213</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>1213</v>
       </c>
       <c r="C40" t="s">
-        <v>1039</v>
+        <v>1204</v>
       </c>
       <c r="D40" t="s">
-        <v>1040</v>
+        <v>1206</v>
       </c>
       <c r="E40" t="s">
-        <v>751</v>
+        <v>1207</v>
       </c>
       <c r="F40" t="s">
-        <v>1040</v>
-      </c>
-      <c r="G40" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>48</v>
       </c>
       <c r="H40" t="s">
-        <v>1041</v>
-      </c>
-      <c r="I40" t="s">
-        <v>7</v>
-      </c>
-      <c r="J40" t="s">
+        <v>1210</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J40" s="6" t="s">
         <v>16</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>1355</v>
+        <v>1352</v>
       </c>
       <c r="M40" t="s">
-        <v>1042</v>
+        <v>1212</v>
       </c>
       <c r="O40" t="s">
-        <v>1043</v>
+        <v>610</v>
       </c>
       <c r="P40" t="s">
         <v>895</v>
@@ -21915,19 +21933,19 @@
         <v>1039</v>
       </c>
       <c r="D41" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="E41" t="s">
         <v>751</v>
       </c>
       <c r="F41" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="G41" t="s">
         <v>48</v>
       </c>
       <c r="H41" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="I41" t="s">
         <v>7</v>
@@ -21936,10 +21954,10 @@
         <v>16</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="M41" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="O41" t="s">
         <v>1043</v>
@@ -21959,19 +21977,19 @@
         <v>1039</v>
       </c>
       <c r="D42" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="E42" t="s">
         <v>751</v>
       </c>
       <c r="F42" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="G42" t="s">
         <v>48</v>
       </c>
       <c r="H42" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="I42" t="s">
         <v>7</v>
@@ -21980,10 +21998,10 @@
         <v>16</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="M42" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="O42" t="s">
         <v>1043</v>
@@ -22003,19 +22021,19 @@
         <v>1039</v>
       </c>
       <c r="D43" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="E43" t="s">
         <v>751</v>
       </c>
       <c r="F43" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="G43" t="s">
         <v>48</v>
       </c>
       <c r="H43" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="I43" t="s">
         <v>7</v>
@@ -22024,10 +22042,10 @@
         <v>16</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="M43" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="O43" t="s">
         <v>1043</v>
@@ -22047,19 +22065,19 @@
         <v>1039</v>
       </c>
       <c r="D44" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="E44" t="s">
         <v>751</v>
       </c>
       <c r="F44" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="G44" t="s">
         <v>48</v>
       </c>
       <c r="H44" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="I44" t="s">
         <v>7</v>
@@ -22068,10 +22086,10 @@
         <v>16</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="M44" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="O44" t="s">
         <v>1043</v>
@@ -22091,19 +22109,19 @@
         <v>1039</v>
       </c>
       <c r="D45" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="E45" t="s">
         <v>751</v>
       </c>
       <c r="F45" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="G45" t="s">
         <v>48</v>
       </c>
       <c r="H45" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="I45" t="s">
         <v>7</v>
@@ -22112,10 +22130,10 @@
         <v>16</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="M45" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
       <c r="O45" t="s">
         <v>1043</v>
@@ -22135,19 +22153,19 @@
         <v>1039</v>
       </c>
       <c r="D46" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="E46" t="s">
         <v>751</v>
       </c>
       <c r="F46" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
       <c r="G46" t="s">
         <v>48</v>
       </c>
       <c r="H46" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="I46" t="s">
         <v>7</v>
@@ -22156,10 +22174,10 @@
         <v>16</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="M46" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="O46" t="s">
         <v>1043</v>
@@ -22179,19 +22197,19 @@
         <v>1039</v>
       </c>
       <c r="D47" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="E47" t="s">
         <v>751</v>
       </c>
       <c r="F47" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="G47" t="s">
         <v>48</v>
       </c>
       <c r="H47" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="I47" t="s">
         <v>7</v>
@@ -22200,10 +22218,10 @@
         <v>16</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="M47" t="s">
-        <v>1064</v>
+        <v>1061</v>
       </c>
       <c r="O47" t="s">
         <v>1043</v>
@@ -22223,19 +22241,19 @@
         <v>1039</v>
       </c>
       <c r="D48" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="E48" t="s">
         <v>751</v>
       </c>
       <c r="F48" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
       <c r="G48" t="s">
         <v>48</v>
       </c>
       <c r="H48" t="s">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="I48" t="s">
         <v>7</v>
@@ -22244,10 +22262,10 @@
         <v>16</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="M48" t="s">
-        <v>1067</v>
+        <v>1064</v>
       </c>
       <c r="O48" t="s">
         <v>1043</v>
@@ -22267,19 +22285,19 @@
         <v>1039</v>
       </c>
       <c r="D49" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="E49" t="s">
         <v>751</v>
       </c>
       <c r="F49" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="G49" t="s">
         <v>48</v>
       </c>
       <c r="H49" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="I49" t="s">
         <v>7</v>
@@ -22288,10 +22306,10 @@
         <v>16</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="M49" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="O49" t="s">
         <v>1043</v>
@@ -22302,28 +22320,28 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>611</v>
+        <v>1037</v>
       </c>
       <c r="B50" t="s">
-        <v>611</v>
+        <v>1038</v>
       </c>
       <c r="C50" t="s">
-        <v>617</v>
+        <v>1039</v>
       </c>
       <c r="D50" t="s">
-        <v>611</v>
+        <v>1068</v>
       </c>
       <c r="E50" t="s">
-        <v>525</v>
+        <v>751</v>
       </c>
       <c r="F50" t="s">
-        <v>611</v>
+        <v>1068</v>
       </c>
       <c r="G50" t="s">
         <v>48</v>
       </c>
       <c r="H50" t="s">
-        <v>616</v>
+        <v>1069</v>
       </c>
       <c r="I50" t="s">
         <v>7</v>
@@ -22331,40 +22349,43 @@
       <c r="J50" t="s">
         <v>16</v>
       </c>
+      <c r="L50" s="6" t="s">
+        <v>1364</v>
+      </c>
       <c r="M50" t="s">
-        <v>878</v>
+        <v>1070</v>
       </c>
       <c r="O50" t="s">
-        <v>618</v>
+        <v>1043</v>
       </c>
       <c r="P50" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>875</v>
+        <v>611</v>
       </c>
       <c r="B51" t="s">
-        <v>875</v>
+        <v>611</v>
       </c>
       <c r="C51" t="s">
-        <v>877</v>
+        <v>617</v>
       </c>
       <c r="D51" t="s">
-        <v>874</v>
+        <v>611</v>
       </c>
       <c r="E51" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="F51" t="s">
-        <v>874</v>
+        <v>611</v>
       </c>
       <c r="G51" t="s">
         <v>48</v>
       </c>
       <c r="H51" t="s">
-        <v>876</v>
+        <v>616</v>
       </c>
       <c r="I51" t="s">
         <v>7</v>
@@ -22373,39 +22394,39 @@
         <v>16</v>
       </c>
       <c r="M51" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="O51" t="s">
         <v>618</v>
       </c>
       <c r="P51" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>887</v>
+        <v>875</v>
       </c>
       <c r="B52" t="s">
-        <v>886</v>
+        <v>875</v>
       </c>
       <c r="C52" t="s">
-        <v>886</v>
+        <v>877</v>
       </c>
       <c r="D52" t="s">
-        <v>880</v>
+        <v>874</v>
       </c>
       <c r="E52" t="s">
         <v>527</v>
       </c>
       <c r="F52" t="s">
-        <v>880</v>
+        <v>874</v>
       </c>
       <c r="G52" t="s">
         <v>48</v>
       </c>
       <c r="H52" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="I52" t="s">
         <v>7</v>
@@ -22414,7 +22435,7 @@
         <v>16</v>
       </c>
       <c r="M52" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="O52" t="s">
         <v>618</v>
@@ -22425,7 +22446,7 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B53" t="s">
         <v>886</v>
@@ -22434,19 +22455,19 @@
         <v>886</v>
       </c>
       <c r="D53" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="E53" t="s">
         <v>527</v>
       </c>
       <c r="F53" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="G53" t="s">
         <v>48</v>
       </c>
       <c r="H53" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="I53" t="s">
         <v>7</v>
@@ -22455,7 +22476,7 @@
         <v>16</v>
       </c>
       <c r="M53" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="O53" t="s">
         <v>618</v>
@@ -22466,28 +22487,28 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>861</v>
+        <v>888</v>
       </c>
       <c r="B54" t="s">
-        <v>861</v>
+        <v>886</v>
       </c>
       <c r="C54" t="s">
-        <v>862</v>
+        <v>886</v>
       </c>
       <c r="D54" t="s">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="E54" t="s">
-        <v>864</v>
+        <v>527</v>
       </c>
       <c r="F54" t="s">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="G54" t="s">
         <v>48</v>
       </c>
       <c r="H54" t="s">
-        <v>865</v>
+        <v>884</v>
       </c>
       <c r="I54" t="s">
         <v>7</v>
@@ -22496,10 +22517,10 @@
         <v>16</v>
       </c>
       <c r="M54" t="s">
-        <v>866</v>
+        <v>885</v>
       </c>
       <c r="O54" t="s">
-        <v>867</v>
+        <v>618</v>
       </c>
       <c r="P54" t="s">
         <v>895</v>
@@ -22507,40 +22528,40 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>930</v>
+        <v>861</v>
       </c>
       <c r="B55" t="s">
-        <v>615</v>
+        <v>861</v>
       </c>
       <c r="C55" t="s">
-        <v>615</v>
+        <v>862</v>
       </c>
       <c r="D55" t="s">
-        <v>931</v>
+        <v>863</v>
       </c>
       <c r="E55" t="s">
-        <v>527</v>
+        <v>864</v>
       </c>
       <c r="F55" t="s">
-        <v>931</v>
+        <v>863</v>
       </c>
       <c r="G55" t="s">
         <v>48</v>
       </c>
       <c r="H55" t="s">
-        <v>932</v>
+        <v>865</v>
       </c>
       <c r="I55" t="s">
         <v>7</v>
       </c>
       <c r="J55" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M55" t="s">
-        <v>934</v>
+        <v>866</v>
       </c>
       <c r="O55" t="s">
-        <v>933</v>
+        <v>867</v>
       </c>
       <c r="P55" t="s">
         <v>895</v>
@@ -22548,40 +22569,40 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>1111</v>
+        <v>930</v>
       </c>
       <c r="B56" t="s">
-        <v>1111</v>
+        <v>615</v>
       </c>
       <c r="C56" t="s">
-        <v>1110</v>
+        <v>615</v>
       </c>
       <c r="D56" t="s">
-        <v>1112</v>
+        <v>931</v>
       </c>
       <c r="E56" t="s">
-        <v>1106</v>
+        <v>527</v>
       </c>
       <c r="F56" t="s">
-        <v>1116</v>
+        <v>931</v>
       </c>
       <c r="G56" t="s">
         <v>48</v>
       </c>
       <c r="H56" t="s">
-        <v>1120</v>
+        <v>932</v>
       </c>
       <c r="I56" t="s">
         <v>7</v>
       </c>
       <c r="J56" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M56" t="s">
-        <v>1109</v>
+        <v>934</v>
       </c>
       <c r="O56" t="s">
-        <v>565</v>
+        <v>933</v>
       </c>
       <c r="P56" t="s">
         <v>895</v>
@@ -22598,19 +22619,19 @@
         <v>1110</v>
       </c>
       <c r="D57" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="E57" t="s">
         <v>1106</v>
       </c>
       <c r="F57" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="G57" t="s">
         <v>48</v>
       </c>
       <c r="H57" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="I57" t="s">
         <v>7</v>
@@ -22639,19 +22660,19 @@
         <v>1110</v>
       </c>
       <c r="D58" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="E58" t="s">
         <v>1106</v>
       </c>
       <c r="F58" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="G58" t="s">
         <v>48</v>
       </c>
       <c r="H58" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="I58" t="s">
         <v>7</v>
@@ -22680,19 +22701,19 @@
         <v>1110</v>
       </c>
       <c r="D59" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="E59" t="s">
         <v>1106</v>
       </c>
       <c r="F59" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="G59" t="s">
         <v>48</v>
       </c>
       <c r="H59" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="I59" t="s">
         <v>7</v>
@@ -22721,19 +22742,19 @@
         <v>1110</v>
       </c>
       <c r="D60" t="s">
-        <v>1105</v>
+        <v>1115</v>
       </c>
       <c r="E60" t="s">
         <v>1106</v>
       </c>
       <c r="F60" t="s">
-        <v>1107</v>
+        <v>1119</v>
       </c>
       <c r="G60" t="s">
         <v>48</v>
       </c>
       <c r="H60" t="s">
-        <v>1108</v>
+        <v>1123</v>
       </c>
       <c r="I60" t="s">
         <v>7</v>
@@ -22753,28 +22774,28 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>556</v>
+        <v>1111</v>
       </c>
       <c r="B61" t="s">
-        <v>562</v>
+        <v>1111</v>
       </c>
       <c r="C61" t="s">
-        <v>562</v>
+        <v>1110</v>
       </c>
       <c r="D61" t="s">
-        <v>556</v>
+        <v>1105</v>
       </c>
       <c r="E61" t="s">
-        <v>557</v>
+        <v>1106</v>
       </c>
       <c r="F61" t="s">
-        <v>556</v>
+        <v>1107</v>
       </c>
       <c r="G61" t="s">
-        <v>558</v>
+        <v>48</v>
       </c>
       <c r="H61" t="s">
-        <v>561</v>
+        <v>1108</v>
       </c>
       <c r="I61" t="s">
         <v>7</v>
@@ -22783,39 +22804,39 @@
         <v>16</v>
       </c>
       <c r="M61" t="s">
-        <v>566</v>
+        <v>1109</v>
       </c>
       <c r="O61" t="s">
         <v>565</v>
       </c>
       <c r="P61" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="B62" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C62" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D62" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="E62" t="s">
         <v>557</v>
       </c>
       <c r="F62" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="G62" t="s">
-        <v>48</v>
+        <v>558</v>
       </c>
       <c r="H62" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="I62" t="s">
         <v>7</v>
@@ -22824,7 +22845,7 @@
         <v>16</v>
       </c>
       <c r="M62" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="O62" t="s">
         <v>565</v>
@@ -22835,28 +22856,28 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>1246</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>1246</v>
+        <v>559</v>
+      </c>
+      <c r="B63" t="s">
+        <v>564</v>
       </c>
       <c r="C63" t="s">
-        <v>1248</v>
+        <v>564</v>
       </c>
       <c r="D63" t="s">
-        <v>1244</v>
+        <v>559</v>
       </c>
       <c r="E63" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="F63" t="s">
-        <v>1244</v>
+        <v>559</v>
       </c>
       <c r="G63" t="s">
         <v>48</v>
       </c>
       <c r="H63" t="s">
-        <v>1245</v>
+        <v>560</v>
       </c>
       <c r="I63" t="s">
         <v>7</v>
@@ -22865,12 +22886,53 @@
         <v>16</v>
       </c>
       <c r="M63" t="s">
+        <v>567</v>
+      </c>
+      <c r="O63" t="s">
+        <v>565</v>
+      </c>
+      <c r="P63" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1244</v>
+      </c>
+      <c r="E64" t="s">
+        <v>527</v>
+      </c>
+      <c r="F64" t="s">
+        <v>1244</v>
+      </c>
+      <c r="G64" t="s">
+        <v>48</v>
+      </c>
+      <c r="H64" t="s">
+        <v>1245</v>
+      </c>
+      <c r="I64" t="s">
+        <v>7</v>
+      </c>
+      <c r="J64" t="s">
+        <v>16</v>
+      </c>
+      <c r="M64" t="s">
         <v>1247</v>
       </c>
-      <c r="O63" t="s">
+      <c r="O64" t="s">
         <v>1243</v>
       </c>
-      <c r="P63" t="s">
+      <c r="P64" t="s">
         <v>895</v>
       </c>
     </row>

</xml_diff>